<commit_message>
Stakeholder workbook: business-facing rewrite of the text (16 review changes)
Scoring date instead of snapshot; RL window from Jan 2019; Unknown and Repeat
delinquent shown with short labels; Step 0 asks "Is the start of this
delinquency missing?" so yes leads to Unknown; months before the current
delinquency instead of months on book; shorter exact tests (stabilized as
short-term / long-term); no "why at this point" column; CC-only worked
examples; thresholds without code names; data handling updated (window start,
history starting overdue, RL first month); "What changed" sheet removed; no
technical wording. P11 updated (7 sheets, --scoring-date).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/deterioration_states/spark/stakeholder/dpd_deterioration_states_reference.xlsx
+++ b/docs/deterioration_states/spark/stakeholder/dpd_deterioration_states_reference.xlsx
@@ -15,7 +15,6 @@
     <sheet name="Buckets &amp; segments" sheetId="5" state="visible" r:id="rId7"/>
     <sheet name="Data handling" sheetId="6" state="visible" r:id="rId8"/>
     <sheet name="Results" sheetId="7" state="visible" r:id="rId9"/>
-    <sheet name="What changed" sheetId="8" state="visible" r:id="rId10"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -27,39 +26,39 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="469" uniqueCount="317">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="420" uniqueCount="284">
   <si>
     <t xml:space="preserve">DPD deterioration states</t>
   </si>
   <si>
-    <t xml:space="preserve">One of the persona axes: how a delinquent account got where it is, read only from its monthly DPD history. Every account in scope gets exactly one of seven states.</t>
+    <t xml:space="preserve">One of the persona axes: how a delinquent account got where it is, read from its monthly DPD history. Every account in scope gets exactly one state.</t>
   </si>
   <si>
     <t xml:space="preserve">Scope</t>
   </si>
   <si>
-    <t xml:space="preserve">Credit cards (CC) and retail loans (RL) at 61–180 DPD and at 180+ DPD on the snapshot date (to be filled from the PROD run). Both segments use the same seven states.</t>
+    <t xml:space="preserve">Credit cards (CC) and retail loans (RL) at 61–180 DPD and at 180+ DPD on the scoring date (to be filled).</t>
   </si>
   <si>
     <t xml:space="preserve">Input</t>
   </si>
   <si>
-    <t xml:space="preserve">One DPD bucket per account per month. CC from Jan 2024 (older history has known data-quality issues); RL full history.</t>
+    <t xml:space="preserve">One DPD bucket per account per month. CC from Jan 2024 (older history has known data-quality issues); RL from Jan 2019.</t>
   </si>
   <si>
     <t xml:space="preserve">How</t>
   </si>
   <si>
-    <t xml:space="preserve">Six yes/no questions asked in a fixed order; the first 'yes' decides the state. See 'How states are assigned'.</t>
+    <t xml:space="preserve">Six yes/no questions in a fixed order; the first 'yes' decides. See 'How states are assigned'.</t>
   </si>
   <si>
     <t xml:space="preserve">Over time</t>
   </si>
   <si>
-    <t xml:space="preserve">Stabilized and EPD describe current behaviour and can change month to month. The others describe how the account fell in and stay fixed — except that any account can move into Stabilized.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The seven states</t>
+    <t xml:space="preserve">EPD and Stabilized can change month to month. The others are fixed once set, except that an account can move into Stabilized.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The states</t>
   </si>
   <si>
     <t xml:space="preserve">State</t>
@@ -77,13 +76,13 @@
     <t xml:space="preserve">Decided at step</t>
   </si>
   <si>
-    <t xml:space="preserve">Unknown — start of the delinquency journey not observed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">We cannot see how the account fell into delinquency: the oldest month we hold is already overdue.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Treat on current behaviour and the other persona axes only.</t>
+    <t xml:space="preserve">Unknown</t>
+  </si>
+  <si>
+    <t xml:space="preserve">We cannot see how the account fell into delinquency: the start of this delinquency is not in the history we hold.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Treat on current behaviour and the other persona axes.</t>
   </si>
   <si>
     <t xml:space="preserve">Fixed</t>
@@ -95,13 +94,13 @@
     <t xml:space="preserve">Early payment default (EPD)</t>
   </si>
   <si>
-    <t xml:space="preserve">Fell behind within its first 3 months on book and has never paid since — still getting worse every month.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Early-risk / first-party fraud review, early legal; no restructuring.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Current — ends the month the customer pays</t>
+    <t xml:space="preserve">Fell behind within 3 months of the start of its history and has not paid since.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Early-risk / first-party fraud review; early legal; no restructuring.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Current: ends when the customer pays</t>
   </si>
   <si>
     <t xml:space="preserve">1</t>
@@ -110,25 +109,25 @@
     <t xml:space="preserve">Stabilized</t>
   </si>
   <si>
-    <t xml:space="preserve">Paying about one month's due each month: the DPD bucket has stopped climbing. Only possible up to 151–180 DPD.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Offer restructuring to break the hardship.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Current — re-read every month</t>
+    <t xml:space="preserve">Paying about one month's due each month: the bucket has stopped climbing. 61–180 DPD only.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Offer restructuring.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Current: re-read monthly</t>
   </si>
   <si>
     <t xml:space="preserve">2</t>
   </si>
   <si>
-    <t xml:space="preserve">Repeat delinquent (re-default)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Was 31+ DPD before, caught up, and fell back in within 12 months.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Has shown they can catch up: firm promise-based plan; credibility decides the pressure.</t>
+    <t xml:space="preserve">Repeat delinquent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Was 31+ DPD before, caught up, and fell back within 12 months.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Firm promise-based plan; credibility sets the pressure.</t>
   </si>
   <si>
     <t xml:space="preserve">3</t>
@@ -137,10 +136,10 @@
     <t xml:space="preserve">Seasoned straight roller</t>
   </si>
   <si>
-    <t xml:space="preserve">On book 12+ months, then missed every payment straight from current to 61+ DPD.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Life event: read with the other axes (departed / income shock / won't pay); most likely to respond to a hardship route.</t>
+    <t xml:space="preserve">Rolled straight to 61+ DPD (no payment), 12+ months after its history began.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Likely a life event: read with the other axes; best fit for a hardship route.</t>
   </si>
   <si>
     <t xml:space="preserve">4</t>
@@ -149,16 +148,16 @@
     <t xml:space="preserve">Early-life straight roller</t>
   </si>
   <si>
-    <t xml:space="preserve">Same straight roll, but in the first 12 months on book (after the EPD window).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Same triage as seasoned; also an underwriting signal for acquisition.</t>
+    <t xml:space="preserve">Rolled straight to 61+ DPD within its first 12 months (after the EPD window).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As seasoned; also an underwriting signal.</t>
   </si>
   <si>
     <t xml:space="preserve">Slow roller (partial payer)</t>
   </si>
   <si>
-    <t xml:space="preserve">Paid something on the way down to 61+ DPD but kept rolling.</t>
+    <t xml:space="preserve">Paid something on the way to 61+ DPD but kept rolling.</t>
   </si>
   <si>
     <t xml:space="preserve">Over-indebted: longer-tenor restructure or settlement.</t>
@@ -167,13 +166,13 @@
     <t xml:space="preserve">5</t>
   </si>
   <si>
-    <t xml:space="preserve">Shares by product and segment: see 'Results'. Thresholds: see 'Thresholds'.</t>
+    <t xml:space="preserve">Shares: see 'Results'. Thresholds: see 'Thresholds'.</t>
   </si>
   <si>
     <t xml:space="preserve">How states are assigned</t>
   </si>
   <si>
-    <t xml:space="preserve">Questions are asked top to bottom. The first 'yes' decides the state, so every account lands in exactly one state. Read the flow first, then the exact tests.</t>
+    <t xml:space="preserve">Questions are asked top to bottom; the first 'yes' decides the state.</t>
   </si>
   <si>
     <t xml:space="preserve">The flow</t>
@@ -182,13 +181,13 @@
     <t xml:space="preserve">Step 0</t>
   </si>
   <si>
-    <t xml:space="preserve">Can we see how the account fell in?</t>
+    <t xml:space="preserve">Is the start of this delinquency missing?</t>
   </si>
   <si>
     <t xml:space="preserve">yes  ▶</t>
   </si>
   <si>
-    <t xml:space="preserve">Unknown  (or Stabilized, if the Step 2 test passes)</t>
+    <t xml:space="preserve">Unknown  (Stabilized if Step 2 passes)</t>
   </si>
   <si>
     <t xml:space="preserve">no  ▼</t>
@@ -218,7 +217,7 @@
     <t xml:space="preserve">Straight roller?</t>
   </si>
   <si>
-    <t xml:space="preserve">Seasoned straight roller  (12+ months on book)</t>
+    <t xml:space="preserve">Seasoned straight roller  (12+ months)</t>
   </si>
   <si>
     <t xml:space="preserve">Early-life straight roller  (&lt; 12 months)</t>
@@ -248,97 +247,78 @@
     <t xml:space="preserve">Exact test</t>
   </si>
   <si>
-    <t xml:space="preserve">Why at this point</t>
-  </si>
-  <si>
-    <t xml:space="preserve">If the OLDEST month we hold is already 1+ DPD, the start of this delinquency is not visible (CC history before Jan 2024 is not used; migrated, restructured or missing history). Such an account is Stabilized if the Step 2 test passes, otherwise Unknown.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Every later step needs the start of the journey; Stabilized needs only the last 6 months.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">All of: at most 3 months on book before first falling 1+ DPD (one short slip that was paid off is allowed); no earlier delinquency; and NOT ONE payment since — every month one bucket worse (months held at the ceiling bucket, CC 210+ / RL 180+, do not count as payments).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Checked before Stabilized so a brand-new non-payer is never read as stable.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Today at most 151–180 DPD (CC bucket ≤ 7, RL ≤ 6) — never in 180+ — AND either 5 of the last 6 months within one bucket of today's, or 6+ months since first reaching 61+ DPD and at most 1 bucket higher than 6 months ago.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Current behaviour wins over how the account fell in: it points to the action.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">An earlier delinquency reached 31+ DPD, was cured, and ended at most 12 months before this one started.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Recent recovery is stronger evidence than the shape of the latest fall.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Went 1–30 → 31–60 → 61–90 DPD in consecutive months (no payment on the way). Seasoned if on book 12+ months before the fall, or if its history starts before Jan 2024 (so it is older than that); otherwise Early-life.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Splits by tenure because the action differs (life event vs underwriting).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Paid at least once on the way down to 61+ DPD but kept rolling.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Everything left: no account is unclassified.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Terms used above</t>
+    <t xml:space="preserve">Oldest month we hold is already overdue (CC 1+ DPD; RL 31+ DPD). Stabilized if Step 2 passes, else Unknown.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fell behind within 3 months of the start of its history, with no earlier delinquency (one short paid-off slip allowed), and has not paid since: one bucket worse every month.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Today 61–180 DPD and no longer getting worse. Either:
+• short-term: in 5 of the last 6 months the bucket was within one of today's; or
+• long-term: 6+ months after reaching 61+ DPD, today's bucket is at most 1 higher than 6 months ago.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">An earlier delinquency reached 31+ DPD, was cured, and ended at most 12 months before this one began.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1–30 → 31–60 → 61–90 DPD in three consecutive months (no payment). Seasoned if 12+ months of history before this delinquency (or history older than the window); otherwise Early-life.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Everything else: paid at least once on the way to 61+ DPD.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Terms</t>
   </si>
   <si>
     <t xml:space="preserve">DPD bucket</t>
   </si>
   <si>
-    <t xml:space="preserve">The account's days-past-due band at month end (see 'Buckets &amp; segments'). One value per month is all the states use.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Delinquency (spell)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A continuous run of months at 1+ DPD. The current spell is the one the account is in today.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Short slip (blip)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">An earlier 1–2 month spell that never passed 1–30 DPD and was paid off. It is not counted as an earlier delinquency.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Month-to-month reading</t>
-  </si>
-  <si>
-    <t xml:space="preserve">One bucket worse = nothing paid (roll). Same bucket = one month's due paid (hold). Better = two or more months paid.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Months on book before the spell</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Months of history before the current spell started.</t>
+    <t xml:space="preserve">Days-past-due band at month end (see 'Buckets &amp; segments').</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Delinquency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A continuous run of months at 1+ DPD.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Short slip</t>
+  </si>
+  <si>
+    <t xml:space="preserve">An earlier 1–2 month delinquency, never past 1–30 DPD, paid off. Not counted as an earlier delinquency.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Month to month</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One bucket worse = nothing paid. Same bucket = one month's due paid. Better = two or more months paid.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Months before this delinquency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Months in the history before the current delinquency started.</t>
   </si>
   <si>
     <t xml:space="preserve">Ceiling bucket</t>
   </si>
   <si>
-    <t xml:space="preserve">The highest bucket: CC 210+ DPD, RL 180+ DPD. It cannot rise, so staying there is not a payment.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cropped history</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Older months exist but are not used (CC before Jan 2024; a long gap in the data). A cropped account is never EPD and counts as seasoned.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Worked examples</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Each row is one account's monthly DPD bucket, oldest on the left, this month on the right. Every example is run through the production rules when this workbook is built.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bucket colours (CC numbering)</t>
+    <t xml:space="preserve">CC 210+ / RL 180+ DPD. The bucket cannot rise, so staying there is not a payment.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">History window</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CC Jan 2024, RL Jan 2019. With older history an account is never EPD, and a straight roller counts as seasoned.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Worked examples (credit cards)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One account per row: monthly DPD bucket, oldest on the left, this month on the right.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bucket colours</t>
   </si>
   <si>
     <t xml:space="preserve">0/1: 0 DPD</t>
@@ -368,9 +348,6 @@
     <t xml:space="preserve">9: 210+</t>
   </si>
   <si>
-    <t xml:space="preserve">Product</t>
-  </si>
-  <si>
     <t xml:space="preserve">-17</t>
   </si>
   <si>
@@ -428,66 +405,54 @@
     <t xml:space="preserve">Why</t>
   </si>
   <si>
-    <t xml:space="preserve">CC</t>
-  </si>
-  <si>
     <t xml:space="preserve">·</t>
   </si>
   <si>
-    <t xml:space="preserve">3 clean months, then one bucket worse every month: never paid.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Same story at 180+: the months held at the ceiling (9 9 9) are not payments.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Holding at 91–120 DPD for 5 months: paying about one month's due.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Swings between 61–90 and 151–180 DPD but no worse than 6 months ago: pays on average. (8 earlier months not shown.)</t>
+    <t xml:space="preserve">3 clean months, then one bucket worse every month.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Same at 180+: months at the ceiling (9 9 9) are not payments.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Holding at 91–120 DPD for 5 months.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Swings between 61–90 and 151–180 DPD, no worse than 6 months ago. (8 earlier months not shown.)</t>
   </si>
   <si>
     <t xml:space="preserve">0 → 2</t>
   </si>
   <si>
-    <t xml:space="preserve">Journey start not visible (delinquent since before Jan 2024), but clearly holding. Older history exists but is not used.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reached 61–90 DPD, caught up fully, fell back in 8 months later.</t>
+    <t xml:space="preserve">Overdue since before Jan 2024, but clearly holding.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reached 61–90 DPD, caught up, fell back 8 months later.</t>
   </si>
   <si>
     <t xml:space="preserve">14 clean months, then missed every payment.</t>
   </si>
   <si>
-    <t xml:space="preserve">Looks short, but its history starts before Jan 2024: older than a year. Older history exists but is not used.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6 clean months (past the EPD window), then a straight roll.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Paid one month at 1–30 and at 31–60 DPD on the way down, still rolled.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Holding at 181–210 DPD is NOT stabilized: Stabilized stops at 151–180 DPD. (6 earlier months not shown.)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Already 121–150 DPD in the oldest month we hold: the fall is not visible. Older history exists but is not used.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Retail loan, RL numbering (1 = 1–30 DPD): reads exactly like the CC case above.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">'·' = no history yet (account not open). RL buckets: 0 = 0 DPD, 1 = 1–30 … 6 = 151–180, 7 = 180+ — coloured like the CC bucket one higher.</t>
+    <t xml:space="preserve">History starts before Jan 2024: older than a year.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6 clean months, then a straight roll.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Paid one month at 1–30 and at 31–60 DPD, still rolled.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Holding at 181–210 DPD is not Stabilized (61–180 DPD only). (6 earlier months not shown.)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Already 121–150 DPD in the oldest month we hold.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">'·' = no history yet (account not open).</t>
   </si>
   <si>
     <t xml:space="preserve">Thresholds</t>
   </si>
   <si>
-    <t xml:space="preserve">The numbers behind the rules, as used by the pipeline. Business thresholds change only with the business owner. Editing a cell here does NOT change the pipeline.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Applies to</t>
   </si>
   <si>
@@ -497,229 +462,196 @@
     <t xml:space="preserve">Value</t>
   </si>
   <si>
-    <t xml:space="preserve">Unit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Why this value</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Name in code</t>
-  </si>
-  <si>
     <t xml:space="preserve">Early payment default</t>
   </si>
   <si>
-    <t xml:space="preserve">Months on book allowed before the first missed payment</t>
-  </si>
-  <si>
-    <t xml:space="preserve">months</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A customer who never pays misses the 1st or 2nd bill: 2–3 clean months at most.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">epd_max_history</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Short paid-off slips allowed before the fall</t>
-  </si>
-  <si>
-    <t xml:space="preserve">slips</t>
-  </si>
-  <si>
-    <t xml:space="preserve">One brief slip that was paid off does not show good behaviour was ever established.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">epd_max_blips</t>
+    <t xml:space="preserve">Months before first falling behind</t>
+  </si>
+  <si>
+    <t xml:space="preserve">≤ 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Someone who never pays misses the 1st or 2nd bill.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Short paid-off slips allowed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One brief slip doesn't show good behaviour.</t>
   </si>
   <si>
     <t xml:space="preserve">Straight roller</t>
   </si>
   <si>
-    <t xml:space="preserve">Months from current to 61–90 DPD to count as a straight roll</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1–30 → 31–60 → 61–90 in consecutive months = no payment on the way.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">straight_max_runup</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Of the last 6 months, how many within one bucket of today's</t>
-  </si>
-  <si>
-    <t xml:space="preserve">of 6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The bank's existing stabilized rule.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">stabilized_min_in_band</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Long-run clause: months since first reaching 61+ DPD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gives an account two full up-down cycles before a plateau counts as stable.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">stabilized_long_run_months</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Long-run clause: at most this many buckets higher than 6 months ago</t>
-  </si>
-  <si>
-    <t xml:space="preserve">bucket</t>
-  </si>
-  <si>
-    <t xml:space="preserve">One bucket of drift is normal; more is still getting worse.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">stabilized_long_run_max_rise</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Highest bucket at which an account can be Stabilized</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CC 7 / RL 6</t>
+    <t xml:space="preserve">Months from first miss to 61–90 DPD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Three misses in a row: nothing paid on the way.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Last 6 months within one bucket of today's</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5 of 6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The bank's existing rule.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stabilized (long-term)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Months since reaching 61+ DPD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gives uneven payers time before a plateau counts.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rise vs 6 months ago</t>
+  </si>
+  <si>
+    <t xml:space="preserve">≤ 1 bucket</t>
+  </si>
+  <si>
+    <t xml:space="preserve">More than one bucket means still getting worse.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Highest DPD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">151–180</t>
+  </si>
+  <si>
+    <t xml:space="preserve">At 180+ a flat bucket is not evidence of payment.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Depth of the earlier delinquency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">31+ DPD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Matches the bank's re-default view.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Months since it ended</t>
+  </si>
+  <si>
+    <t xml:space="preserve">≤ 12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Common re-default window.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seasoned vs early-life</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Standard first-year window.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CC data used from</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jan 2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Older CC data has known quality issues.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RL data used from</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jan 2019</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Start of the RL window.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Missing months</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Filled if the gap is at most</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 months</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Longer gaps: history starts after the gap.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buckets &amp; segments</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CC and RL number buckets differently; the rules read both as DPD bands.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DPD band</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CC bucket</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RL bucket</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Segment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Note</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0 DPD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0 (no due) / 1 (current)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">—</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clean.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1–30 DPD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Delinquency starts.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">31–60 DPD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">61–90 DPD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">61–180 DPD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Segment starts.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">91–120 DPD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">121–150 DPD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6</t>
   </si>
   <si>
     <t xml:space="preserve">151–180 DPD</t>
   </si>
   <si>
-    <t xml:space="preserve">At 180+ staying in the same bucket is not evidence of payment.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">stabilized_max_bucket</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Repeat delinquent</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Depth the earlier delinquency must have reached</t>
-  </si>
-  <si>
-    <t xml:space="preserve">31–60 DPD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cures from 61+ DPD are rare; 31+ DPD matches the bank's own re-default view.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">repeat_min_prior_peak</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Months between the earlier cure and the new fall</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The common re-default window.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">repeat_window_months</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Seasoned vs early-life</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Months on book before the fall to count as seasoned</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Standard first-year early-life window; EPD already takes the first 3 months.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">seasoned_min_months</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Data (CC only)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Billing history used from</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jan 2024</t>
-  </si>
-  <si>
-    <t xml:space="preserve">date</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Older CC history has known data-quality issues (temporary).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cc_history_floor_date</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Data</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Missing months filled by inference if the gap is at most</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Longer gaps: history starts after the gap (see 'Data handling').</t>
-  </si>
-  <si>
-    <t xml:space="preserve">max_inferred_gap_months</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Buckets &amp; segments</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CC and RL number their buckets differently; the rules are the same once both are read as DPD bands.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DPD band</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CC bucket</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RL bucket</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Segment</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Note</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0 DPD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0 (no due) / 1 (current)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">—</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Clean.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1–30 DPD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Delinquency starts here.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">61–90 DPD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">61–180 DPD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Spine starts here.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">91–120 DPD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">121–150 DPD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6</t>
-  </si>
-  <si>
     <t xml:space="preserve">7</t>
   </si>
   <si>
-    <t xml:space="preserve">Highest bucket at which Stabilized is possible.</t>
+    <t xml:space="preserve">Highest bucket for Stabilized.</t>
   </si>
   <si>
     <t xml:space="preserve">181–210 DPD</t>
@@ -734,7 +666,7 @@
     <t xml:space="preserve">180+ DPD</t>
   </si>
   <si>
-    <t xml:space="preserve">RL ceiling: RL 7 covers all of 180+.</t>
+    <t xml:space="preserve">RL ceiling: RL 7 = all of 180+.</t>
   </si>
   <si>
     <t xml:space="preserve">210+ DPD</t>
@@ -743,13 +675,13 @@
     <t xml:space="preserve">9 (ceiling)</t>
   </si>
   <si>
-    <t xml:space="preserve">CC ceiling. Staying at the ceiling is not a payment.</t>
+    <t xml:space="preserve">CC ceiling.</t>
   </si>
   <si>
     <t xml:space="preserve">Reading one month to the next</t>
   </si>
   <si>
-    <t xml:space="preserve">Bucket this month vs last</t>
+    <t xml:space="preserve">This month vs last</t>
   </si>
   <si>
     <t xml:space="preserve">Meaning</t>
@@ -761,19 +693,19 @@
     <t xml:space="preserve">One bucket worse</t>
   </si>
   <si>
-    <t xml:space="preserve">Roll — nothing paid</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Same bucket (below the ceiling)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hold — one month's due paid</t>
+    <t xml:space="preserve">Nothing paid</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Same bucket</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One month's due paid</t>
   </si>
   <si>
     <t xml:space="preserve">k buckets better</t>
   </si>
   <si>
-    <t xml:space="preserve">Paid k + 1 months at once</t>
+    <t xml:space="preserve">k + 1 months paid at once</t>
   </si>
   <si>
     <t xml:space="preserve">k + 1</t>
@@ -782,22 +714,22 @@
     <t xml:space="preserve">Back to 0 DPD</t>
   </si>
   <si>
-    <t xml:space="preserve">Cure — rare from 61+ DPD</t>
+    <t xml:space="preserve">Cured (rare from 61+ DPD)</t>
   </si>
   <si>
     <t xml:space="preserve">all</t>
   </si>
   <si>
-    <t xml:space="preserve">Same bucket AT the ceiling</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Unknown — the bucket cannot rise; NOT a payment</t>
+    <t xml:space="preserve">Same bucket at the ceiling</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not a payment: the bucket cannot rise</t>
   </si>
   <si>
     <t xml:space="preserve">Data handling</t>
   </si>
   <si>
-    <t xml:space="preserve">How the monthly history is prepared before the questions are asked. Nothing is dropped silently; every fix is counted per account.</t>
+    <t xml:space="preserve">How the monthly history is prepared before the questions are asked.</t>
   </si>
   <si>
     <t xml:space="preserve">Situation</t>
@@ -806,49 +738,64 @@
     <t xml:space="preserve">What we do</t>
   </si>
   <si>
-    <t xml:space="preserve">Effect on the states</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CC history before Jan 2024</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Not used (known data-quality issue, temporary).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The account's history is 'cropped': never EPD; a straight roller counts as seasoned; if the oldest month we hold is overdue → Unknown (unless Stabilized).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Two bills in one month, none in the next</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Billing-cycle shift: one bill is moved to the empty month.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">None — restores the true monthly sequence.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A missing month between two equal buckets</t>
+    <t xml:space="preserve">Effect on states</t>
+  </si>
+  <si>
+    <t xml:space="preserve">History before the window start (CC Jan 2024, RL Jan 2019)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not used.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Never EPD; a straight roller counts as seasoned.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">History starts already overdue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Start of the delinquency is missing.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unknown, unless Stabilized.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RL loan 1–30 DPD in its first month</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Normal: its first payment is due that month.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Classified as usual.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Two bills in one month, none in the next (CC)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One bill moved to the empty month.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">None.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Missing month between two equal buckets</t>
   </si>
   <si>
     <t xml:space="preserve">Filled with that bucket.</t>
   </si>
   <si>
-    <t xml:space="preserve">None.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A missing month where only a straight roll fits (3 _ 5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Filled as the roll (3 4 5).</t>
+    <t xml:space="preserve">Missing month where only a straight roll fits</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Filled as the roll.</t>
   </si>
   <si>
     <t xml:space="preserve">Other gaps of up to 2 months</t>
   </si>
   <si>
-    <t xml:space="preserve">Filled: last known bucket carried, rising as late as possible.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Can read as a payment (hold); counted per account.</t>
+    <t xml:space="preserve">Filled: last bucket carried, rising as late as possible.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Can read as a payment.</t>
   </si>
   <si>
     <t xml:space="preserve">Longer gaps</t>
@@ -857,40 +804,40 @@
     <t xml:space="preserve">History starts after the gap.</t>
   </si>
   <si>
-    <t xml:space="preserve">Treated like cropped history.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Impossible one-month blips (4 0 4, 0 3 0)</t>
+    <t xml:space="preserve">As for history before the window start.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One-month blips (4 0 4, 0 3 0)</t>
   </si>
   <si>
     <t xml:space="preserve">Corrected to the neighbours.</t>
   </si>
   <si>
-    <t xml:space="preserve">Prevents a false cure or a false earlier delinquency.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Billing-cycle jumps (3 3 5 / 3 5 5 for 3 4 5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Corrected to the straight roll.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prevents a false payment.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No bucket on any row / no bill in the window</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Account kept with a status, not classified.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reported as lost coverage (target: 99.9% classified).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Last month older than the snapshot</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Flagged (months stale).</t>
+    <t xml:space="preserve">No false cure or false earlier delinquency.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Billing-cycle jumps (3 3 5 for 3 4 5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Corrected to the roll.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No false payment.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No usable bucket in the window</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not classified.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Counts against coverage (target 99.9%).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Latest month older than the scoring date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flagged.</t>
   </si>
   <si>
     <t xml:space="preserve">Classified on the history we have.</t>
@@ -899,7 +846,7 @@
     <t xml:space="preserve">Results</t>
   </si>
   <si>
-    <t xml:space="preserve">Accounts per state (PROD run, snapshot to be filled from the PROD run). Blue numbers come from the PROD check (prod_check.report(catalog, save_json=...)); shares and coverage are formulas. Yellow = still to fill in.</t>
+    <t xml:space="preserve">Accounts per state, scoring date to be filled. Blue = counts from the scoring run; shares and coverage are calculated. Yellow = to fill in.</t>
   </si>
   <si>
     <t xml:space="preserve">CC 61–180 DPD
@@ -930,58 +877,13 @@
     <t xml:space="preserve">Coverage (target 99.9%)</t>
   </si>
   <si>
-    <t xml:space="preserve">Stabilized cannot occur at 180+ by design (Stabilized stops at 151–180 DPD).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Roll rates are not shown: measured on the same months that define a state they are circular (EPD rolls 100% by definition). Forward-looking outcomes come from the backtest.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Aggregates only: no account ids, no DPD histories.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">What changed since the 16 Oct 2026 version</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Change</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Retail loans and the 180+ segment added, with the same seven states as CC 61–180.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">One vocabulary for every product and segment.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">'Not classified — history starts delinquent' is now 'Unknown' and also covers accounts already overdue in the oldest month we hold (e.g. delinquent since before Jan 2024).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">When the start of the journey is not visible, how the account fell in would be a guess.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stabilized only up to 151–180 DPD; never at 180+.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Months held at the ceiling bucket (CC 210+, RL 180+) are not payments.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keeps EPD meaningful at 180+.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The live 'Rule tester' sheet is replaced by worked examples computed by the production rules.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The formulas were a second copy of the rules and had drifted (no Unknown, no 180+ rule).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Roll rate removed from the results.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">It was measured on the same months that define the states (EPD = 100% by definition).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thresholds shown with plain names; parameter names kept in a side column.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Readable for the business; traceable to the code.</t>
+    <t xml:space="preserve">Stabilized is not possible at 180+ (61–180 DPD only).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Roll rates are not shown: they would be measured on the same months that define the states.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No account-level data.</t>
   </si>
 </sst>
 </file>
@@ -994,7 +896,7 @@
     <numFmt numFmtId="166" formatCode="0.0%"/>
     <numFmt numFmtId="167" formatCode="0.00%"/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="20">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1126,13 +1028,6 @@
     <font>
       <sz val="10"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="8"/>
-      <color rgb="FF595959"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -1328,7 +1223,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="64">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1521,10 +1416,6 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="10" fillId="11" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1565,7 +1456,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="20" fillId="19" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="19" fillId="19" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1581,7 +1472,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="20" fillId="19" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="19" fillId="19" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1904,7 +1795,7 @@
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="58"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="50"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="24"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="12"/>
   </cols>
@@ -1923,7 +1814,7 @@
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
     </row>
-    <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -1934,7 +1825,7 @@
       <c r="D4" s="4"/>
       <c r="E4" s="4"/>
     </row>
-    <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
         <v>4</v>
       </c>
@@ -1945,7 +1836,7 @@
       <c r="D5" s="4"/>
       <c r="E5" s="4"/>
     </row>
-    <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
         <v>6</v>
       </c>
@@ -1956,7 +1847,7 @@
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
     </row>
-    <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
         <v>8</v>
       </c>
@@ -1993,7 +1884,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="8" t="s">
         <v>16</v>
       </c>
@@ -2010,7 +1901,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="11" t="s">
         <v>21</v>
       </c>
@@ -2027,7 +1918,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="12" t="s">
         <v>26</v>
       </c>
@@ -2044,7 +1935,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
         <v>31</v>
       </c>
@@ -2061,7 +1952,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="14" t="s">
         <v>35</v>
       </c>
@@ -2078,7 +1969,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="15" t="s">
         <v>39</v>
       </c>
@@ -2095,7 +1986,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="16" t="s">
         <v>42</v>
       </c>
@@ -2140,14 +2031,14 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="44"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2163,7 +2054,6 @@
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
@@ -2173,7 +2063,6 @@
       <c r="C4" s="6"/>
       <c r="D4" s="6"/>
       <c r="E4" s="6"/>
-      <c r="F4" s="6"/>
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
@@ -2295,9 +2184,8 @@
       <c r="C17" s="6"/>
       <c r="D17" s="6"/>
       <c r="E17" s="6"/>
-      <c r="F17" s="6"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
         <v>69</v>
       </c>
@@ -2311,11 +2199,8 @@
         <v>72</v>
       </c>
       <c r="E18" s="7"/>
-      <c r="F18" s="7" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="19" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="10" t="s">
         <v>20</v>
       </c>
@@ -2326,14 +2211,11 @@
         <v>16</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E19" s="9"/>
-      <c r="F19" s="9" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="20" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="10" t="s">
         <v>25</v>
       </c>
@@ -2344,14 +2226,11 @@
         <v>21</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="E20" s="9"/>
-      <c r="F20" s="9" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="21" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="10" t="s">
         <v>30</v>
       </c>
@@ -2362,14 +2241,11 @@
         <v>26</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="E21" s="9"/>
-      <c r="F21" s="9" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="22" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="10" t="s">
         <v>34</v>
       </c>
@@ -2380,14 +2256,11 @@
         <v>31</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="E22" s="9"/>
-      <c r="F22" s="9" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="23" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="s">
         <v>38</v>
       </c>
@@ -2398,14 +2271,11 @@
         <v>35</v>
       </c>
       <c r="D23" s="9" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="E23" s="9"/>
-      <c r="F23" s="9" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="66" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="24" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="10" t="s">
         <v>45</v>
       </c>
@@ -2416,110 +2286,100 @@
         <v>42</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="E24" s="9"/>
-      <c r="F24" s="9" t="s">
-        <v>85</v>
-      </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="B26" s="6"/>
       <c r="C26" s="6"/>
       <c r="D26" s="6"/>
       <c r="E26" s="6"/>
-      <c r="F26" s="6"/>
-    </row>
-    <row r="27" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="27" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="22" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="B27" s="22"/>
       <c r="C27" s="4" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="D27" s="4"/>
       <c r="E27" s="4"/>
-      <c r="F27" s="4"/>
-    </row>
-    <row r="28" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="28" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="22" t="s">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="B28" s="22"/>
       <c r="C28" s="4" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="D28" s="4"/>
       <c r="E28" s="4"/>
-      <c r="F28" s="4"/>
-    </row>
-    <row r="29" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="29" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="22" t="s">
-        <v>91</v>
+        <v>84</v>
       </c>
       <c r="B29" s="22"/>
       <c r="C29" s="4" t="s">
-        <v>92</v>
+        <v>85</v>
       </c>
       <c r="D29" s="4"/>
       <c r="E29" s="4"/>
-      <c r="F29" s="4"/>
-    </row>
-    <row r="30" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="30" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="22" t="s">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="B30" s="22"/>
       <c r="C30" s="4" t="s">
-        <v>94</v>
+        <v>87</v>
       </c>
       <c r="D30" s="4"/>
       <c r="E30" s="4"/>
-      <c r="F30" s="4"/>
-    </row>
-    <row r="31" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="31" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="22" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="B31" s="22"/>
       <c r="C31" s="4" t="s">
-        <v>96</v>
+        <v>89</v>
       </c>
       <c r="D31" s="4"/>
       <c r="E31" s="4"/>
-      <c r="F31" s="4"/>
-    </row>
-    <row r="32" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="32" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="22" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="B32" s="22"/>
       <c r="C32" s="4" t="s">
-        <v>98</v>
+        <v>91</v>
       </c>
       <c r="D32" s="4"/>
       <c r="E32" s="4"/>
-      <c r="F32" s="4"/>
-    </row>
-    <row r="33" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="33" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="22" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="B33" s="22"/>
       <c r="C33" s="4" t="s">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="D33" s="4"/>
       <c r="E33" s="4"/>
-      <c r="F33" s="4"/>
     </row>
   </sheetData>
-  <mergeCells count="21">
-    <mergeCell ref="A2:F2"/>
+  <mergeCells count="22">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="D18:E18"/>
     <mergeCell ref="D19:E19"/>
     <mergeCell ref="D20:E20"/>
     <mergeCell ref="D21:E21"/>
@@ -2527,19 +2387,19 @@
     <mergeCell ref="D23:E23"/>
     <mergeCell ref="D24:E24"/>
     <mergeCell ref="A27:B27"/>
-    <mergeCell ref="C27:F27"/>
+    <mergeCell ref="C27:E27"/>
     <mergeCell ref="A28:B28"/>
-    <mergeCell ref="C28:F28"/>
+    <mergeCell ref="C28:E28"/>
     <mergeCell ref="A29:B29"/>
-    <mergeCell ref="C29:F29"/>
+    <mergeCell ref="C29:E29"/>
     <mergeCell ref="A30:B30"/>
-    <mergeCell ref="C30:F30"/>
+    <mergeCell ref="C30:E30"/>
     <mergeCell ref="A31:B31"/>
-    <mergeCell ref="C31:F31"/>
+    <mergeCell ref="C31:E31"/>
     <mergeCell ref="A32:B32"/>
-    <mergeCell ref="C32:F32"/>
+    <mergeCell ref="C32:E32"/>
     <mergeCell ref="A33:B33"/>
-    <mergeCell ref="C33:F33"/>
+    <mergeCell ref="C33:E33"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2556,25 +2416,24 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:W21"/>
+  <dimension ref="A1:V20"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="4" style="0" width="5.2"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="0" width="48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="3" style="0" width="5.2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="0" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="0" width="6"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2597,160 +2456,156 @@
       <c r="T2" s="2"/>
       <c r="U2" s="2"/>
       <c r="V2" s="2"/>
-      <c r="W2" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="23" t="s">
+        <v>96</v>
+      </c>
+      <c r="C4" s="24" t="s">
+        <v>97</v>
+      </c>
+      <c r="D4" s="24"/>
+      <c r="E4" s="25" t="s">
+        <v>98</v>
+      </c>
+      <c r="F4" s="25"/>
+      <c r="G4" s="26" t="s">
+        <v>99</v>
+      </c>
+      <c r="H4" s="26"/>
+      <c r="I4" s="27" t="s">
+        <v>100</v>
+      </c>
+      <c r="J4" s="27"/>
+      <c r="K4" s="28" t="s">
+        <v>101</v>
+      </c>
+      <c r="L4" s="28"/>
+      <c r="M4" s="29" t="s">
+        <v>102</v>
+      </c>
+      <c r="N4" s="29"/>
+      <c r="O4" s="30" t="s">
         <v>103</v>
       </c>
-      <c r="D4" s="24" t="s">
+      <c r="P4" s="30"/>
+      <c r="Q4" s="31" t="s">
         <v>104</v>
       </c>
-      <c r="E4" s="24"/>
-      <c r="F4" s="25" t="s">
+      <c r="R4" s="31"/>
+      <c r="S4" s="32" t="s">
         <v>105</v>
       </c>
-      <c r="G4" s="25"/>
-      <c r="H4" s="26" t="s">
-        <v>106</v>
-      </c>
-      <c r="I4" s="26"/>
-      <c r="J4" s="27" t="s">
-        <v>107</v>
-      </c>
-      <c r="K4" s="27"/>
-      <c r="L4" s="28" t="s">
-        <v>108</v>
-      </c>
-      <c r="M4" s="28"/>
-      <c r="N4" s="29" t="s">
-        <v>109</v>
-      </c>
-      <c r="O4" s="29"/>
-      <c r="P4" s="30" t="s">
-        <v>110</v>
-      </c>
-      <c r="Q4" s="30"/>
-      <c r="R4" s="31" t="s">
-        <v>111</v>
-      </c>
-      <c r="S4" s="31"/>
-      <c r="T4" s="32" t="s">
-        <v>112</v>
-      </c>
-      <c r="U4" s="32"/>
+      <c r="T4" s="32"/>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
         <v>11</v>
       </c>
       <c r="B6" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="I6" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="J6" s="7" t="s">
         <v>113</v>
       </c>
-      <c r="C6" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="D6" s="7" t="s">
+      <c r="K6" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="L6" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="M6" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="G6" s="7" t="s">
+      <c r="N6" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="H6" s="7" t="s">
+      <c r="O6" s="7" t="s">
         <v>118</v>
       </c>
-      <c r="I6" s="7" t="s">
+      <c r="P6" s="7" t="s">
         <v>119</v>
       </c>
-      <c r="J6" s="7" t="s">
+      <c r="Q6" s="7" t="s">
         <v>120</v>
       </c>
-      <c r="K6" s="7" t="s">
+      <c r="R6" s="7" t="s">
         <v>121</v>
       </c>
-      <c r="L6" s="7" t="s">
+      <c r="S6" s="7" t="s">
         <v>122</v>
       </c>
-      <c r="M6" s="7" t="s">
+      <c r="T6" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="N6" s="7" t="s">
+      <c r="U6" s="7" t="s">
         <v>124</v>
       </c>
-      <c r="O6" s="7" t="s">
-        <v>125</v>
-      </c>
-      <c r="P6" s="7" t="s">
-        <v>126</v>
-      </c>
-      <c r="Q6" s="7" t="s">
-        <v>127</v>
-      </c>
-      <c r="R6" s="7" t="s">
-        <v>128</v>
-      </c>
-      <c r="S6" s="7" t="s">
-        <v>129</v>
-      </c>
-      <c r="T6" s="7" t="s">
-        <v>130</v>
-      </c>
-      <c r="U6" s="7" t="s">
-        <v>131</v>
-      </c>
-      <c r="V6" s="7" t="s">
-        <v>132</v>
-      </c>
-      <c r="W6" s="7"/>
-    </row>
-    <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="V6" s="7"/>
+    </row>
+    <row r="7" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="11" t="s">
         <v>21</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>133</v>
-      </c>
-      <c r="C7" s="10" t="s">
         <v>25</v>
       </c>
+      <c r="C7" s="33" t="s">
+        <v>125</v>
+      </c>
       <c r="D7" s="33" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="E7" s="33" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="F7" s="33" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="G7" s="33" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="H7" s="33" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="I7" s="33" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="J7" s="33" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="K7" s="33" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="L7" s="33" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="M7" s="33" t="s">
-        <v>134</v>
-      </c>
-      <c r="N7" s="33" t="s">
-        <v>134</v>
+        <v>125</v>
+      </c>
+      <c r="N7" s="34" t="n">
+        <v>0</v>
       </c>
       <c r="O7" s="34" t="n">
         <v>0</v>
@@ -2758,107 +2613,101 @@
       <c r="P7" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="Q7" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="R7" s="35" t="n">
+      <c r="Q7" s="35" t="n">
         <v>2</v>
       </c>
-      <c r="S7" s="36" t="n">
+      <c r="R7" s="36" t="n">
         <v>3</v>
       </c>
-      <c r="T7" s="37" t="n">
+      <c r="S7" s="37" t="n">
         <v>4</v>
       </c>
-      <c r="U7" s="38" t="n">
+      <c r="T7" s="38" t="n">
         <v>5</v>
       </c>
-      <c r="V7" s="9" t="s">
-        <v>135</v>
-      </c>
-      <c r="W7" s="9"/>
-    </row>
-    <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="U7" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="V7" s="9"/>
+    </row>
+    <row r="8" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
         <v>21</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>133</v>
-      </c>
-      <c r="C8" s="10" t="s">
         <v>25</v>
       </c>
+      <c r="C8" s="33" t="s">
+        <v>125</v>
+      </c>
       <c r="D8" s="33" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="E8" s="33" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="F8" s="33" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="G8" s="33" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="H8" s="33" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="I8" s="33" t="s">
-        <v>134</v>
-      </c>
-      <c r="J8" s="33" t="s">
-        <v>134</v>
-      </c>
-      <c r="K8" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="L8" s="35" t="n">
+        <v>125</v>
+      </c>
+      <c r="J8" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="35" t="n">
         <v>2</v>
       </c>
-      <c r="M8" s="36" t="n">
+      <c r="L8" s="36" t="n">
         <v>3</v>
       </c>
-      <c r="N8" s="37" t="n">
+      <c r="M8" s="37" t="n">
         <v>4</v>
       </c>
-      <c r="O8" s="39" t="n">
+      <c r="N8" s="39" t="n">
         <v>5</v>
       </c>
-      <c r="P8" s="40" t="n">
+      <c r="O8" s="40" t="n">
         <v>6</v>
       </c>
-      <c r="Q8" s="41" t="n">
+      <c r="P8" s="41" t="n">
         <v>7</v>
       </c>
-      <c r="R8" s="42" t="n">
+      <c r="Q8" s="42" t="n">
         <v>8</v>
+      </c>
+      <c r="R8" s="43" t="n">
+        <v>9</v>
       </c>
       <c r="S8" s="43" t="n">
         <v>9</v>
       </c>
-      <c r="T8" s="43" t="n">
+      <c r="T8" s="44" t="n">
         <v>9</v>
       </c>
-      <c r="U8" s="44" t="n">
-        <v>9</v>
-      </c>
-      <c r="V8" s="9" t="s">
-        <v>136</v>
-      </c>
-      <c r="W8" s="9"/>
-    </row>
-    <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="U8" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="V8" s="9"/>
+    </row>
+    <row r="9" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="12" t="s">
         <v>26</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>133</v>
-      </c>
-      <c r="C9" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="D9" s="33" t="s">
-        <v>134</v>
+      <c r="C9" s="33" t="s">
+        <v>125</v>
+      </c>
+      <c r="D9" s="34" t="n">
+        <v>0</v>
       </c>
       <c r="E9" s="34" t="n">
         <v>0</v>
@@ -2881,20 +2730,20 @@
       <c r="K9" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="L9" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="M9" s="35" t="n">
+      <c r="L9" s="35" t="n">
         <v>2</v>
       </c>
-      <c r="N9" s="36" t="n">
+      <c r="M9" s="36" t="n">
         <v>3</v>
+      </c>
+      <c r="N9" s="37" t="n">
+        <v>4</v>
       </c>
       <c r="O9" s="37" t="n">
         <v>4</v>
       </c>
-      <c r="P9" s="37" t="n">
-        <v>4</v>
+      <c r="P9" s="39" t="n">
+        <v>5</v>
       </c>
       <c r="Q9" s="39" t="n">
         <v>5</v>
@@ -2905,32 +2754,29 @@
       <c r="S9" s="39" t="n">
         <v>5</v>
       </c>
-      <c r="T9" s="39" t="n">
+      <c r="T9" s="38" t="n">
         <v>5</v>
       </c>
-      <c r="U9" s="38" t="n">
-        <v>5</v>
-      </c>
-      <c r="V9" s="9" t="s">
-        <v>137</v>
-      </c>
-      <c r="W9" s="9"/>
-    </row>
-    <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="U9" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="V9" s="9"/>
+    </row>
+    <row r="10" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="12" t="s">
         <v>26</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>133</v>
-      </c>
-      <c r="C10" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="D10" s="35" t="n">
+      <c r="C10" s="35" t="n">
         <v>2</v>
       </c>
-      <c r="E10" s="36" t="n">
+      <c r="D10" s="36" t="n">
         <v>3</v>
+      </c>
+      <c r="E10" s="37" t="n">
+        <v>4</v>
       </c>
       <c r="F10" s="37" t="n">
         <v>4</v>
@@ -2938,63 +2784,58 @@
       <c r="G10" s="37" t="n">
         <v>4</v>
       </c>
-      <c r="H10" s="37" t="n">
-        <v>4</v>
+      <c r="H10" s="36" t="n">
+        <v>3</v>
       </c>
       <c r="I10" s="36" t="n">
         <v>3</v>
       </c>
-      <c r="J10" s="36" t="n">
+      <c r="J10" s="37" t="n">
+        <v>4</v>
+      </c>
+      <c r="K10" s="39" t="n">
+        <v>5</v>
+      </c>
+      <c r="L10" s="37" t="n">
+        <v>4</v>
+      </c>
+      <c r="M10" s="36" t="n">
         <v>3</v>
-      </c>
-      <c r="K10" s="37" t="n">
-        <v>4</v>
-      </c>
-      <c r="L10" s="39" t="n">
-        <v>5</v>
-      </c>
-      <c r="M10" s="37" t="n">
-        <v>4</v>
       </c>
       <c r="N10" s="36" t="n">
         <v>3</v>
       </c>
-      <c r="O10" s="36" t="n">
-        <v>3</v>
-      </c>
-      <c r="P10" s="37" t="n">
+      <c r="O10" s="37" t="n">
         <v>4</v>
       </c>
-      <c r="Q10" s="39" t="n">
+      <c r="P10" s="39" t="n">
         <v>5</v>
       </c>
-      <c r="R10" s="40" t="n">
+      <c r="Q10" s="40" t="n">
         <v>6</v>
+      </c>
+      <c r="R10" s="39" t="n">
+        <v>5</v>
       </c>
       <c r="S10" s="39" t="n">
         <v>5</v>
       </c>
-      <c r="T10" s="39" t="n">
-        <v>5</v>
-      </c>
-      <c r="U10" s="45" t="n">
+      <c r="T10" s="45" t="n">
         <v>4</v>
       </c>
-      <c r="V10" s="9" t="s">
-        <v>138</v>
-      </c>
-      <c r="W10" s="9"/>
-    </row>
-    <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="U10" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="V10" s="9"/>
+    </row>
+    <row r="11" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="12" t="s">
         <v>26</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>133</v>
-      </c>
-      <c r="C11" s="10" t="s">
-        <v>139</v>
-      </c>
+        <v>130</v>
+      </c>
+      <c r="C11" s="33"/>
       <c r="D11" s="33"/>
       <c r="E11" s="33"/>
       <c r="F11" s="33"/>
@@ -3006,7 +2847,9 @@
       <c r="L11" s="33"/>
       <c r="M11" s="33"/>
       <c r="N11" s="33"/>
-      <c r="O11" s="33"/>
+      <c r="O11" s="39" t="n">
+        <v>5</v>
+      </c>
       <c r="P11" s="39" t="n">
         <v>5</v>
       </c>
@@ -3019,45 +2862,42 @@
       <c r="S11" s="39" t="n">
         <v>5</v>
       </c>
-      <c r="T11" s="39" t="n">
+      <c r="T11" s="38" t="n">
         <v>5</v>
       </c>
-      <c r="U11" s="38" t="n">
-        <v>5</v>
-      </c>
-      <c r="V11" s="9" t="s">
-        <v>140</v>
-      </c>
-      <c r="W11" s="9"/>
-    </row>
-    <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="U11" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="V11" s="9"/>
+    </row>
+    <row r="12" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
         <v>31</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>133</v>
-      </c>
-      <c r="C12" s="10" t="s">
         <v>34</v>
       </c>
+      <c r="C12" s="33" t="s">
+        <v>125</v>
+      </c>
       <c r="D12" s="33" t="s">
-        <v>134</v>
-      </c>
-      <c r="E12" s="33" t="s">
-        <v>134</v>
-      </c>
-      <c r="F12" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="G12" s="35" t="n">
+        <v>125</v>
+      </c>
+      <c r="E12" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="35" t="n">
         <v>2</v>
       </c>
-      <c r="H12" s="36" t="n">
+      <c r="G12" s="36" t="n">
         <v>3</v>
       </c>
-      <c r="I12" s="37" t="n">
+      <c r="H12" s="37" t="n">
         <v>4</v>
       </c>
+      <c r="I12" s="34" t="n">
+        <v>0</v>
+      </c>
       <c r="J12" s="34" t="n">
         <v>0</v>
       </c>
@@ -3079,105 +2919,97 @@
       <c r="P12" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="Q12" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="R12" s="35" t="n">
+      <c r="Q12" s="35" t="n">
         <v>2</v>
       </c>
-      <c r="S12" s="36" t="n">
+      <c r="R12" s="36" t="n">
         <v>3</v>
       </c>
-      <c r="T12" s="37" t="n">
+      <c r="S12" s="37" t="n">
         <v>4</v>
       </c>
-      <c r="U12" s="38" t="n">
+      <c r="T12" s="38" t="n">
         <v>5</v>
       </c>
-      <c r="V12" s="9" t="s">
-        <v>141</v>
-      </c>
-      <c r="W12" s="9"/>
-    </row>
-    <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="U12" s="9" t="s">
+        <v>132</v>
+      </c>
+      <c r="V12" s="9"/>
+    </row>
+    <row r="13" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="14" t="s">
         <v>35</v>
       </c>
       <c r="B13" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="C13" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="P13" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="R13" s="36" t="n">
+        <v>3</v>
+      </c>
+      <c r="S13" s="37" t="n">
+        <v>4</v>
+      </c>
+      <c r="T13" s="38" t="n">
+        <v>5</v>
+      </c>
+      <c r="U13" s="9" t="s">
         <v>133</v>
       </c>
-      <c r="C13" s="10" t="s">
-        <v>38</v>
-      </c>
-      <c r="D13" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="G13" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="I13" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="J13" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="K13" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="L13" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="M13" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="N13" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="O13" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="P13" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q13" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="R13" s="35" t="n">
-        <v>2</v>
-      </c>
-      <c r="S13" s="36" t="n">
-        <v>3</v>
-      </c>
-      <c r="T13" s="37" t="n">
-        <v>4</v>
-      </c>
-      <c r="U13" s="38" t="n">
-        <v>5</v>
-      </c>
-      <c r="V13" s="9" t="s">
-        <v>142</v>
-      </c>
-      <c r="W13" s="9"/>
-    </row>
-    <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="V13" s="9"/>
+    </row>
+    <row r="14" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="14" t="s">
         <v>35</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>133</v>
-      </c>
-      <c r="C14" s="10" t="s">
         <v>38</v>
       </c>
+      <c r="C14" s="33"/>
       <c r="D14" s="33"/>
       <c r="E14" s="33"/>
       <c r="F14" s="33"/>
@@ -3189,63 +3021,62 @@
       <c r="L14" s="33"/>
       <c r="M14" s="33"/>
       <c r="N14" s="33"/>
-      <c r="O14" s="33"/>
+      <c r="O14" s="34" t="n">
+        <v>0</v>
+      </c>
       <c r="P14" s="34" t="n">
         <v>0</v>
       </c>
       <c r="Q14" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="R14" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="S14" s="35" t="n">
+      <c r="R14" s="35" t="n">
         <v>2</v>
       </c>
-      <c r="T14" s="36" t="n">
+      <c r="S14" s="36" t="n">
         <v>3</v>
       </c>
-      <c r="U14" s="45" t="n">
+      <c r="T14" s="45" t="n">
         <v>4</v>
       </c>
-      <c r="V14" s="9" t="s">
-        <v>143</v>
-      </c>
-      <c r="W14" s="9"/>
-    </row>
-    <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="U14" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="V14" s="9"/>
+    </row>
+    <row r="15" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="15" t="s">
         <v>39</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>133</v>
-      </c>
-      <c r="C15" s="10" t="s">
         <v>38</v>
       </c>
+      <c r="C15" s="33" t="s">
+        <v>125</v>
+      </c>
       <c r="D15" s="33" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="E15" s="33" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="F15" s="33" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="G15" s="33" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="H15" s="33" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="I15" s="33" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="J15" s="33" t="s">
-        <v>134</v>
-      </c>
-      <c r="K15" s="33" t="s">
-        <v>134</v>
+        <v>125</v>
+      </c>
+      <c r="K15" s="34" t="n">
+        <v>0</v>
       </c>
       <c r="L15" s="34" t="n">
         <v>0</v>
@@ -3262,41 +3093,38 @@
       <c r="P15" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="Q15" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="R15" s="35" t="n">
+      <c r="Q15" s="35" t="n">
         <v>2</v>
       </c>
-      <c r="S15" s="36" t="n">
+      <c r="R15" s="36" t="n">
         <v>3</v>
       </c>
-      <c r="T15" s="37" t="n">
+      <c r="S15" s="37" t="n">
         <v>4</v>
       </c>
-      <c r="U15" s="38" t="n">
+      <c r="T15" s="38" t="n">
         <v>5</v>
       </c>
-      <c r="V15" s="9" t="s">
-        <v>144</v>
-      </c>
-      <c r="W15" s="9"/>
-    </row>
-    <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="U15" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="V15" s="9"/>
+    </row>
+    <row r="16" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="16" t="s">
         <v>42</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>133</v>
-      </c>
-      <c r="C16" s="10" t="s">
         <v>45</v>
       </c>
+      <c r="C16" s="33" t="s">
+        <v>125</v>
+      </c>
       <c r="D16" s="33" t="s">
-        <v>134</v>
-      </c>
-      <c r="E16" s="33" t="s">
-        <v>134</v>
+        <v>125</v>
+      </c>
+      <c r="E16" s="34" t="n">
+        <v>0</v>
       </c>
       <c r="F16" s="34" t="n">
         <v>0</v>
@@ -3325,42 +3153,39 @@
       <c r="N16" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="O16" s="34" t="n">
-        <v>0</v>
+      <c r="O16" s="35" t="n">
+        <v>2</v>
       </c>
       <c r="P16" s="35" t="n">
         <v>2</v>
       </c>
-      <c r="Q16" s="35" t="n">
-        <v>2</v>
+      <c r="Q16" s="36" t="n">
+        <v>3</v>
       </c>
       <c r="R16" s="36" t="n">
         <v>3</v>
       </c>
-      <c r="S16" s="36" t="n">
-        <v>3</v>
-      </c>
-      <c r="T16" s="37" t="n">
+      <c r="S16" s="37" t="n">
         <v>4</v>
       </c>
-      <c r="U16" s="38" t="n">
+      <c r="T16" s="38" t="n">
         <v>5</v>
       </c>
-      <c r="V16" s="9" t="s">
-        <v>145</v>
-      </c>
-      <c r="W16" s="9"/>
-    </row>
-    <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="U16" s="9" t="s">
+        <v>136</v>
+      </c>
+      <c r="V16" s="9"/>
+    </row>
+    <row r="17" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="14" t="s">
         <v>35</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>133</v>
-      </c>
-      <c r="C17" s="10" t="s">
         <v>38</v>
       </c>
+      <c r="C17" s="34" t="n">
+        <v>0</v>
+      </c>
       <c r="D17" s="34" t="n">
         <v>0</v>
       </c>
@@ -3376,26 +3201,26 @@
       <c r="H17" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="I17" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="J17" s="35" t="n">
+      <c r="I17" s="35" t="n">
         <v>2</v>
       </c>
-      <c r="K17" s="36" t="n">
+      <c r="J17" s="36" t="n">
         <v>3</v>
       </c>
-      <c r="L17" s="37" t="n">
+      <c r="K17" s="37" t="n">
         <v>4</v>
       </c>
-      <c r="M17" s="39" t="n">
+      <c r="L17" s="39" t="n">
         <v>5</v>
       </c>
-      <c r="N17" s="40" t="n">
+      <c r="M17" s="40" t="n">
         <v>6</v>
       </c>
-      <c r="O17" s="41" t="n">
+      <c r="N17" s="41" t="n">
         <v>7</v>
+      </c>
+      <c r="O17" s="42" t="n">
+        <v>8</v>
       </c>
       <c r="P17" s="42" t="n">
         <v>8</v>
@@ -3409,27 +3234,22 @@
       <c r="S17" s="42" t="n">
         <v>8</v>
       </c>
-      <c r="T17" s="42" t="n">
+      <c r="T17" s="46" t="n">
         <v>8</v>
       </c>
-      <c r="U17" s="46" t="n">
-        <v>8</v>
-      </c>
-      <c r="V17" s="9" t="s">
-        <v>146</v>
-      </c>
-      <c r="W17" s="9"/>
-    </row>
-    <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="U17" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="V17" s="9"/>
+    </row>
+    <row r="18" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="8" t="s">
         <v>16</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>133</v>
-      </c>
-      <c r="C18" s="10" t="s">
         <v>20</v>
       </c>
+      <c r="C18" s="33"/>
       <c r="D18" s="33"/>
       <c r="E18" s="33"/>
       <c r="F18" s="33"/>
@@ -3441,130 +3261,59 @@
       <c r="L18" s="33"/>
       <c r="M18" s="33"/>
       <c r="N18" s="33"/>
-      <c r="O18" s="33"/>
+      <c r="O18" s="40" t="n">
+        <v>6</v>
+      </c>
       <c r="P18" s="40" t="n">
         <v>6</v>
       </c>
-      <c r="Q18" s="40" t="n">
-        <v>6</v>
+      <c r="Q18" s="41" t="n">
+        <v>7</v>
       </c>
       <c r="R18" s="41" t="n">
         <v>7</v>
       </c>
-      <c r="S18" s="41" t="n">
-        <v>7</v>
-      </c>
-      <c r="T18" s="42" t="n">
+      <c r="S18" s="42" t="n">
         <v>8</v>
       </c>
-      <c r="U18" s="44" t="n">
+      <c r="T18" s="44" t="n">
         <v>9</v>
       </c>
-      <c r="V18" s="9" t="s">
-        <v>147</v>
-      </c>
-      <c r="W18" s="9"/>
-    </row>
-    <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="B19" s="10" t="s">
-        <v>148</v>
-      </c>
-      <c r="C19" s="10" t="s">
-        <v>38</v>
-      </c>
-      <c r="D19" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="E19" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="F19" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="G19" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="H19" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="I19" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="J19" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="K19" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="L19" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="M19" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="N19" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="O19" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="P19" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q19" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="R19" s="35" t="n">
-        <v>1</v>
-      </c>
-      <c r="S19" s="36" t="n">
-        <v>2</v>
-      </c>
-      <c r="T19" s="37" t="n">
-        <v>3</v>
-      </c>
-      <c r="U19" s="38" t="n">
-        <v>4</v>
-      </c>
-      <c r="V19" s="9" t="s">
-        <v>149</v>
-      </c>
-      <c r="W19" s="9"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="17" t="s">
-        <v>150</v>
+      <c r="U18" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="V18" s="9"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="17" t="s">
+        <v>139</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="24">
-    <mergeCell ref="A2:W2"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="H4:I4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="L4:M4"/>
-    <mergeCell ref="N4:O4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="R4:S4"/>
-    <mergeCell ref="T4:U4"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="V7:W7"/>
-    <mergeCell ref="V8:W8"/>
-    <mergeCell ref="V9:W9"/>
-    <mergeCell ref="V10:W10"/>
-    <mergeCell ref="V11:W11"/>
-    <mergeCell ref="V12:W12"/>
-    <mergeCell ref="V13:W13"/>
-    <mergeCell ref="V14:W14"/>
-    <mergeCell ref="V15:W15"/>
-    <mergeCell ref="V16:W16"/>
-    <mergeCell ref="V17:W17"/>
-    <mergeCell ref="V18:W18"/>
-    <mergeCell ref="V19:W19"/>
+  <mergeCells count="23">
+    <mergeCell ref="A2:V2"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="I4:J4"/>
+    <mergeCell ref="K4:L4"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="O4:P4"/>
+    <mergeCell ref="Q4:R4"/>
+    <mergeCell ref="S4:T4"/>
+    <mergeCell ref="U6:V6"/>
+    <mergeCell ref="U7:V7"/>
+    <mergeCell ref="U8:V8"/>
+    <mergeCell ref="U9:V9"/>
+    <mergeCell ref="U10:V10"/>
+    <mergeCell ref="U11:V11"/>
+    <mergeCell ref="U12:V12"/>
+    <mergeCell ref="U13:V13"/>
+    <mergeCell ref="U14:V14"/>
+    <mergeCell ref="U15:V15"/>
+    <mergeCell ref="U16:V16"/>
+    <mergeCell ref="U17:V17"/>
+    <mergeCell ref="U18:V18"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -3581,295 +3330,217 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="50"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="54"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>142</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="9" t="s">
+        <v>144</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="C4" s="47" t="s">
+        <v>146</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="9" t="s">
+        <v>144</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>148</v>
+      </c>
+      <c r="C5" s="47" t="s">
+        <v>25</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="B6" s="9" t="s">
         <v>151</v>
       </c>
-    </row>
-    <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="C6" s="47" t="s">
+        <v>34</v>
+      </c>
+      <c r="D6" s="9" t="s">
         <v>152</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="s">
+    </row>
+    <row r="7" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7" s="9" t="s">
         <v>153</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="C7" s="47" t="s">
         <v>154</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="D7" s="9" t="s">
         <v>155</v>
       </c>
-      <c r="D4" s="7" t="s">
+    </row>
+    <row r="8" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="9" t="s">
         <v>156</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="B8" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="C8" s="47" t="s">
         <v>158</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="9" t="s">
+      <c r="D8" s="9" t="s">
         <v>159</v>
       </c>
-      <c r="B5" s="9" t="s">
+    </row>
+    <row r="9" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="9" t="s">
+        <v>156</v>
+      </c>
+      <c r="B9" s="9" t="s">
         <v>160</v>
       </c>
-      <c r="C5" s="47" t="n">
-        <v>3</v>
-      </c>
-      <c r="D5" s="9" t="s">
+      <c r="C9" s="47" t="s">
         <v>161</v>
       </c>
-      <c r="E5" s="9" t="s">
+      <c r="D9" s="9" t="s">
         <v>162</v>
       </c>
-      <c r="F5" s="48" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="9" t="s">
-        <v>159</v>
-      </c>
-      <c r="B6" s="9" t="s">
-        <v>164</v>
-      </c>
-      <c r="C6" s="47" t="n">
-        <v>1</v>
-      </c>
-      <c r="D6" s="9" t="s">
-        <v>165</v>
-      </c>
-      <c r="E6" s="9" t="s">
-        <v>166</v>
-      </c>
-      <c r="F6" s="48" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="9" t="s">
-        <v>168</v>
-      </c>
-      <c r="B7" s="9" t="s">
-        <v>169</v>
-      </c>
-      <c r="C7" s="47" t="n">
-        <v>3</v>
-      </c>
-      <c r="D7" s="9" t="s">
-        <v>161</v>
-      </c>
-      <c r="E7" s="9" t="s">
-        <v>170</v>
-      </c>
-      <c r="F7" s="48" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>172</v>
-      </c>
-      <c r="C8" s="47" t="n">
-        <v>5</v>
-      </c>
-      <c r="D8" s="9" t="s">
-        <v>173</v>
-      </c>
-      <c r="E8" s="9" t="s">
-        <v>174</v>
-      </c>
-      <c r="F8" s="48" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="B9" s="9" t="s">
-        <v>176</v>
-      </c>
-      <c r="C9" s="47" t="n">
-        <v>6</v>
-      </c>
-      <c r="D9" s="9" t="s">
-        <v>161</v>
-      </c>
-      <c r="E9" s="9" t="s">
-        <v>177</v>
-      </c>
-      <c r="F9" s="48" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="10" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="9" t="s">
         <v>26</v>
       </c>
       <c r="B10" s="9" t="s">
+        <v>163</v>
+      </c>
+      <c r="C10" s="47" t="s">
+        <v>164</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>166</v>
+      </c>
+      <c r="C11" s="47" t="s">
+        <v>167</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>169</v>
+      </c>
+      <c r="C12" s="47" t="s">
+        <v>170</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="9" t="s">
+        <v>172</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="C13" s="47" t="s">
+        <v>173</v>
+      </c>
+      <c r="D13" s="9" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>175</v>
+      </c>
+      <c r="C14" s="47" t="s">
+        <v>176</v>
+      </c>
+      <c r="D14" s="9" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>178</v>
+      </c>
+      <c r="C15" s="47" t="s">
         <v>179</v>
       </c>
-      <c r="C10" s="47" t="n">
-        <v>1</v>
-      </c>
-      <c r="D10" s="9" t="s">
+      <c r="D15" s="9" t="s">
         <v>180</v>
       </c>
-      <c r="E10" s="9" t="s">
+    </row>
+    <row r="16" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="9" t="s">
         <v>181</v>
       </c>
-      <c r="F10" s="48" t="s">
+      <c r="B16" s="9" t="s">
         <v>182</v>
       </c>
-    </row>
-    <row r="11" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="B11" s="9" t="s">
+      <c r="C16" s="47" t="s">
         <v>183</v>
       </c>
-      <c r="C11" s="47" t="s">
+      <c r="D16" s="9" t="s">
         <v>184</v>
       </c>
-      <c r="D11" s="9" t="s">
-        <v>185</v>
-      </c>
-      <c r="E11" s="9" t="s">
-        <v>186</v>
-      </c>
-      <c r="F11" s="48" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="9" t="s">
-        <v>188</v>
-      </c>
-      <c r="B12" s="9" t="s">
-        <v>189</v>
-      </c>
-      <c r="C12" s="47" t="s">
-        <v>190</v>
-      </c>
-      <c r="D12" s="9" t="s">
-        <v>180</v>
-      </c>
-      <c r="E12" s="9" t="s">
-        <v>191</v>
-      </c>
-      <c r="F12" s="48" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="9" t="s">
-        <v>188</v>
-      </c>
-      <c r="B13" s="9" t="s">
-        <v>193</v>
-      </c>
-      <c r="C13" s="47" t="n">
-        <v>12</v>
-      </c>
-      <c r="D13" s="9" t="s">
-        <v>161</v>
-      </c>
-      <c r="E13" s="9" t="s">
-        <v>194</v>
-      </c>
-      <c r="F13" s="48" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="9" t="s">
-        <v>196</v>
-      </c>
-      <c r="B14" s="9" t="s">
-        <v>197</v>
-      </c>
-      <c r="C14" s="47" t="n">
-        <v>12</v>
-      </c>
-      <c r="D14" s="9" t="s">
-        <v>161</v>
-      </c>
-      <c r="E14" s="9" t="s">
-        <v>198</v>
-      </c>
-      <c r="F14" s="48" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="9" t="s">
-        <v>200</v>
-      </c>
-      <c r="B15" s="9" t="s">
-        <v>201</v>
-      </c>
-      <c r="C15" s="47" t="s">
-        <v>202</v>
-      </c>
-      <c r="D15" s="9" t="s">
-        <v>203</v>
-      </c>
-      <c r="E15" s="9" t="s">
-        <v>204</v>
-      </c>
-      <c r="F15" s="48" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="9" t="s">
-        <v>206</v>
-      </c>
-      <c r="B16" s="9" t="s">
-        <v>207</v>
-      </c>
-      <c r="C16" s="47" t="n">
-        <v>2</v>
-      </c>
-      <c r="D16" s="9" t="s">
-        <v>161</v>
-      </c>
-      <c r="E16" s="9" t="s">
-        <v>208</v>
-      </c>
-      <c r="F16" s="48" t="s">
-        <v>209</v>
-      </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A2:F2"/>
-  </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -3888,21 +3559,21 @@
   <dimension ref="A1:E21"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="36"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>210</v>
+        <v>185</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>211</v>
+        <v>186</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -3911,41 +3582,41 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>212</v>
+        <v>187</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>213</v>
+        <v>188</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>214</v>
+        <v>189</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>215</v>
+        <v>190</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>216</v>
+        <v>191</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="49" t="s">
-        <v>217</v>
+      <c r="A5" s="48" t="s">
+        <v>192</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>218</v>
+        <v>193</v>
       </c>
       <c r="C5" s="10" t="s">
         <v>20</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>219</v>
+        <v>194</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>220</v>
+        <v>195</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="50" t="s">
-        <v>221</v>
+      <c r="A6" s="49" t="s">
+        <v>196</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>30</v>
@@ -3954,15 +3625,15 @@
         <v>25</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>219</v>
+        <v>194</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>222</v>
+        <v>197</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="51" t="s">
-        <v>190</v>
+      <c r="A7" s="50" t="s">
+        <v>198</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>34</v>
@@ -3971,13 +3642,13 @@
         <v>30</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>219</v>
+        <v>194</v>
       </c>
       <c r="E7" s="9"/>
     </row>
     <row r="8" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="52" t="s">
-        <v>223</v>
+      <c r="A8" s="51" t="s">
+        <v>199</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>38</v>
@@ -3986,15 +3657,15 @@
         <v>34</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>224</v>
+        <v>200</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>225</v>
+        <v>201</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="53" t="s">
-        <v>226</v>
+      <c r="A9" s="52" t="s">
+        <v>202</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>45</v>
@@ -4003,79 +3674,79 @@
         <v>38</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>224</v>
+        <v>200</v>
       </c>
       <c r="E9" s="9"/>
     </row>
     <row r="10" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="54" t="s">
-        <v>227</v>
+      <c r="A10" s="53" t="s">
+        <v>203</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>228</v>
+        <v>204</v>
       </c>
       <c r="C10" s="10" t="s">
         <v>45</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>224</v>
+        <v>200</v>
       </c>
       <c r="E10" s="9"/>
     </row>
     <row r="11" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="55" t="s">
-        <v>185</v>
+      <c r="A11" s="54" t="s">
+        <v>205</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>229</v>
+        <v>206</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>228</v>
+        <v>204</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>224</v>
+        <v>200</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>230</v>
+        <v>207</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="56" t="s">
-        <v>231</v>
+      <c r="A12" s="55" t="s">
+        <v>208</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>232</v>
+        <v>209</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>233</v>
+        <v>210</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>234</v>
+        <v>211</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>235</v>
+        <v>212</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="57" t="s">
-        <v>236</v>
+      <c r="A13" s="56" t="s">
+        <v>213</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>237</v>
+        <v>214</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>233</v>
+        <v>210</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>234</v>
+        <v>211</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>238</v>
+        <v>215</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>239</v>
+        <v>216</v>
       </c>
       <c r="B15" s="6"/>
       <c r="C15" s="6"/>
@@ -4084,68 +3755,68 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>240</v>
+        <v>217</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>241</v>
+        <v>218</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>243</v>
+        <v>220</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>244</v>
+        <v>221</v>
       </c>
       <c r="C17" s="10" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="9" t="s">
-        <v>245</v>
+        <v>222</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>246</v>
+        <v>223</v>
       </c>
       <c r="C18" s="10" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="9" t="s">
-        <v>247</v>
+        <v>224</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>248</v>
+        <v>225</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="9" t="s">
-        <v>250</v>
+        <v>227</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>251</v>
+        <v>228</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="9" t="s">
-        <v>253</v>
+        <v>230</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>254</v>
+        <v>231</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>219</v>
+        <v>194</v>
       </c>
     </row>
   </sheetData>
@@ -4167,145 +3838,166 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="44"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>255</v>
+        <v>232</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>256</v>
+        <v>233</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
+        <v>234</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>235</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="57" t="s">
+        <v>237</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>238</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="57" t="s">
+        <v>240</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>241</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="57" t="s">
+        <v>243</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="57" t="s">
+        <v>246</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>247</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="57" t="s">
+        <v>249</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>250</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="57" t="s">
+        <v>251</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>252</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="57" t="s">
+        <v>253</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>254</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="57" t="s">
+        <v>256</v>
+      </c>
+      <c r="B12" s="9" t="s">
         <v>257</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="C12" s="9" t="s">
         <v>258</v>
       </c>
-      <c r="C4" s="7" t="s">
+    </row>
+    <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="57" t="s">
         <v>259</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="58" t="s">
+      <c r="B13" s="9" t="s">
         <v>260</v>
       </c>
-      <c r="B5" s="9" t="s">
+      <c r="C13" s="9" t="s">
         <v>261</v>
       </c>
-      <c r="C5" s="9" t="s">
+    </row>
+    <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="57" t="s">
         <v>262</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="58" t="s">
+      <c r="B14" s="9" t="s">
         <v>263</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="C14" s="9" t="s">
         <v>264</v>
       </c>
-      <c r="C6" s="9" t="s">
+    </row>
+    <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="57" t="s">
         <v>265</v>
       </c>
-    </row>
-    <row r="7" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="58" t="s">
+      <c r="B15" s="9" t="s">
         <v>266</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="C15" s="9" t="s">
         <v>267</v>
       </c>
-      <c r="C7" s="9" t="s">
+    </row>
+    <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="57" t="s">
         <v>268</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="58" t="s">
+      <c r="B16" s="9" t="s">
         <v>269</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="C16" s="9" t="s">
         <v>270</v>
-      </c>
-      <c r="C8" s="9" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="58" t="s">
-        <v>271</v>
-      </c>
-      <c r="B9" s="9" t="s">
-        <v>272</v>
-      </c>
-      <c r="C9" s="9" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="58" t="s">
-        <v>274</v>
-      </c>
-      <c r="B10" s="9" t="s">
-        <v>275</v>
-      </c>
-      <c r="C10" s="9" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="58" t="s">
-        <v>277</v>
-      </c>
-      <c r="B11" s="9" t="s">
-        <v>278</v>
-      </c>
-      <c r="C11" s="9" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="58" t="s">
-        <v>280</v>
-      </c>
-      <c r="B12" s="9" t="s">
-        <v>281</v>
-      </c>
-      <c r="C12" s="9" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="58" t="s">
-        <v>283</v>
-      </c>
-      <c r="B13" s="9" t="s">
-        <v>284</v>
-      </c>
-      <c r="C13" s="9" t="s">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="58" t="s">
-        <v>286</v>
-      </c>
-      <c r="B14" s="9" t="s">
-        <v>287</v>
-      </c>
-      <c r="C14" s="9" t="s">
-        <v>288</v>
       </c>
     </row>
   </sheetData>
@@ -4343,12 +4035,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>289</v>
+        <v>271</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>290</v>
+        <v>272</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -4364,51 +4056,51 @@
         <v>11</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>291</v>
+        <v>273</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>292</v>
+        <v>274</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>293</v>
+        <v>275</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>292</v>
+        <v>274</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>294</v>
+        <v>276</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>292</v>
+        <v>274</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>295</v>
+        <v>277</v>
       </c>
       <c r="I4" s="7" t="s">
-        <v>292</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="B5" s="59"/>
-      <c r="C5" s="60" t="str">
+      <c r="B5" s="58"/>
+      <c r="C5" s="59" t="str">
         <f aca="false">IF($B$12=0,"",B5/$B$12)</f>
         <v/>
       </c>
-      <c r="D5" s="59"/>
-      <c r="E5" s="60" t="str">
+      <c r="D5" s="58"/>
+      <c r="E5" s="59" t="str">
         <f aca="false">IF($D$12=0,"",D5/$D$12)</f>
         <v/>
       </c>
-      <c r="F5" s="59"/>
-      <c r="G5" s="60" t="str">
+      <c r="F5" s="58"/>
+      <c r="G5" s="59" t="str">
         <f aca="false">IF($F$12=0,"",F5/$F$12)</f>
         <v/>
       </c>
-      <c r="H5" s="59"/>
-      <c r="I5" s="60" t="str">
+      <c r="H5" s="58"/>
+      <c r="I5" s="59" t="str">
         <f aca="false">IF($H$12=0,"",H5/$H$12)</f>
         <v/>
       </c>
@@ -4417,23 +4109,23 @@
       <c r="A6" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="B6" s="59"/>
-      <c r="C6" s="60" t="str">
+      <c r="B6" s="58"/>
+      <c r="C6" s="59" t="str">
         <f aca="false">IF($B$12=0,"",B6/$B$12)</f>
         <v/>
       </c>
-      <c r="D6" s="59"/>
-      <c r="E6" s="60" t="str">
+      <c r="D6" s="58"/>
+      <c r="E6" s="59" t="str">
         <f aca="false">IF($D$12=0,"",D6/$D$12)</f>
         <v/>
       </c>
-      <c r="F6" s="59"/>
-      <c r="G6" s="60" t="str">
+      <c r="F6" s="58"/>
+      <c r="G6" s="59" t="str">
         <f aca="false">IF($F$12=0,"",F6/$F$12)</f>
         <v/>
       </c>
-      <c r="H6" s="59"/>
-      <c r="I6" s="60" t="str">
+      <c r="H6" s="58"/>
+      <c r="I6" s="59" t="str">
         <f aca="false">IF($H$12=0,"",H6/$H$12)</f>
         <v/>
       </c>
@@ -4442,23 +4134,23 @@
       <c r="A7" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="B7" s="59"/>
-      <c r="C7" s="60" t="str">
+      <c r="B7" s="58"/>
+      <c r="C7" s="59" t="str">
         <f aca="false">IF($B$12=0,"",B7/$B$12)</f>
         <v/>
       </c>
-      <c r="D7" s="59"/>
-      <c r="E7" s="60" t="str">
+      <c r="D7" s="58"/>
+      <c r="E7" s="59" t="str">
         <f aca="false">IF($D$12=0,"",D7/$D$12)</f>
         <v/>
       </c>
-      <c r="F7" s="59"/>
-      <c r="G7" s="60" t="str">
+      <c r="F7" s="58"/>
+      <c r="G7" s="59" t="str">
         <f aca="false">IF($F$12=0,"",F7/$F$12)</f>
         <v/>
       </c>
-      <c r="H7" s="59"/>
-      <c r="I7" s="60" t="str">
+      <c r="H7" s="58"/>
+      <c r="I7" s="59" t="str">
         <f aca="false">IF($H$12=0,"",H7/$H$12)</f>
         <v/>
       </c>
@@ -4467,23 +4159,23 @@
       <c r="A8" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="B8" s="59"/>
-      <c r="C8" s="60" t="str">
+      <c r="B8" s="58"/>
+      <c r="C8" s="59" t="str">
         <f aca="false">IF($B$12=0,"",B8/$B$12)</f>
         <v/>
       </c>
-      <c r="D8" s="59"/>
-      <c r="E8" s="60" t="str">
+      <c r="D8" s="58"/>
+      <c r="E8" s="59" t="str">
         <f aca="false">IF($D$12=0,"",D8/$D$12)</f>
         <v/>
       </c>
-      <c r="F8" s="59"/>
-      <c r="G8" s="60" t="str">
+      <c r="F8" s="58"/>
+      <c r="G8" s="59" t="str">
         <f aca="false">IF($F$12=0,"",F8/$F$12)</f>
         <v/>
       </c>
-      <c r="H8" s="59"/>
-      <c r="I8" s="60" t="str">
+      <c r="H8" s="58"/>
+      <c r="I8" s="59" t="str">
         <f aca="false">IF($H$12=0,"",H8/$H$12)</f>
         <v/>
       </c>
@@ -4492,23 +4184,23 @@
       <c r="A9" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="B9" s="59"/>
-      <c r="C9" s="60" t="str">
+      <c r="B9" s="58"/>
+      <c r="C9" s="59" t="str">
         <f aca="false">IF($B$12=0,"",B9/$B$12)</f>
         <v/>
       </c>
-      <c r="D9" s="59"/>
-      <c r="E9" s="60" t="str">
+      <c r="D9" s="58"/>
+      <c r="E9" s="59" t="str">
         <f aca="false">IF($D$12=0,"",D9/$D$12)</f>
         <v/>
       </c>
-      <c r="F9" s="59"/>
-      <c r="G9" s="60" t="str">
+      <c r="F9" s="58"/>
+      <c r="G9" s="59" t="str">
         <f aca="false">IF($F$12=0,"",F9/$F$12)</f>
         <v/>
       </c>
-      <c r="H9" s="59"/>
-      <c r="I9" s="60" t="str">
+      <c r="H9" s="58"/>
+      <c r="I9" s="59" t="str">
         <f aca="false">IF($H$12=0,"",H9/$H$12)</f>
         <v/>
       </c>
@@ -4517,23 +4209,23 @@
       <c r="A10" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="B10" s="59"/>
-      <c r="C10" s="60" t="str">
+      <c r="B10" s="58"/>
+      <c r="C10" s="59" t="str">
         <f aca="false">IF($B$12=0,"",B10/$B$12)</f>
         <v/>
       </c>
-      <c r="D10" s="59"/>
-      <c r="E10" s="60" t="str">
+      <c r="D10" s="58"/>
+      <c r="E10" s="59" t="str">
         <f aca="false">IF($D$12=0,"",D10/$D$12)</f>
         <v/>
       </c>
-      <c r="F10" s="59"/>
-      <c r="G10" s="60" t="str">
+      <c r="F10" s="58"/>
+      <c r="G10" s="59" t="str">
         <f aca="false">IF($F$12=0,"",F10/$F$12)</f>
         <v/>
       </c>
-      <c r="H10" s="59"/>
-      <c r="I10" s="60" t="str">
+      <c r="H10" s="58"/>
+      <c r="I10" s="59" t="str">
         <f aca="false">IF($H$12=0,"",H10/$H$12)</f>
         <v/>
       </c>
@@ -4542,81 +4234,81 @@
       <c r="A11" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="B11" s="59"/>
-      <c r="C11" s="60" t="str">
+      <c r="B11" s="58"/>
+      <c r="C11" s="59" t="str">
         <f aca="false">IF($B$12=0,"",B11/$B$12)</f>
         <v/>
       </c>
-      <c r="D11" s="59"/>
-      <c r="E11" s="60" t="str">
+      <c r="D11" s="58"/>
+      <c r="E11" s="59" t="str">
         <f aca="false">IF($D$12=0,"",D11/$D$12)</f>
         <v/>
       </c>
-      <c r="F11" s="59"/>
-      <c r="G11" s="60" t="str">
+      <c r="F11" s="58"/>
+      <c r="G11" s="59" t="str">
         <f aca="false">IF($F$12=0,"",F11/$F$12)</f>
         <v/>
       </c>
-      <c r="H11" s="59"/>
-      <c r="I11" s="60" t="str">
+      <c r="H11" s="58"/>
+      <c r="I11" s="59" t="str">
         <f aca="false">IF($H$12=0,"",H11/$H$12)</f>
         <v/>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="23" t="s">
-        <v>296</v>
-      </c>
-      <c r="B12" s="61" t="n">
+        <v>278</v>
+      </c>
+      <c r="B12" s="60" t="n">
         <f aca="false">SUM(B5:B11)</f>
         <v>0</v>
       </c>
-      <c r="D12" s="61" t="n">
+      <c r="D12" s="60" t="n">
         <f aca="false">SUM(D5:D11)</f>
         <v>0</v>
       </c>
-      <c r="F12" s="61" t="n">
+      <c r="F12" s="60" t="n">
         <f aca="false">SUM(F5:F11)</f>
         <v>0</v>
       </c>
-      <c r="H12" s="61" t="n">
+      <c r="H12" s="60" t="n">
         <f aca="false">SUM(H5:H11)</f>
         <v>0</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="62" t="s">
-        <v>297</v>
-      </c>
-      <c r="B13" s="63"/>
-      <c r="D13" s="63"/>
-      <c r="F13" s="63"/>
-      <c r="H13" s="63"/>
+      <c r="A13" s="61" t="s">
+        <v>279</v>
+      </c>
+      <c r="B13" s="62"/>
+      <c r="D13" s="62"/>
+      <c r="F13" s="62"/>
+      <c r="H13" s="62"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="23" t="s">
-        <v>298</v>
-      </c>
-      <c r="B14" s="64" t="str">
+        <v>280</v>
+      </c>
+      <c r="B14" s="63" t="str">
         <f aca="false">IF((B12+B13)=0,"",B12/(B12+B13))</f>
         <v/>
       </c>
-      <c r="D14" s="64" t="str">
+      <c r="D14" s="63" t="str">
         <f aca="false">IF((D12+D13)=0,"",D12/(D12+D13))</f>
         <v/>
       </c>
-      <c r="F14" s="64" t="str">
+      <c r="F14" s="63" t="str">
         <f aca="false">IF((F12+F13)=0,"",F12/(F12+F13))</f>
         <v/>
       </c>
-      <c r="H14" s="64" t="str">
+      <c r="H14" s="63" t="str">
         <f aca="false">IF((H12+H13)=0,"",H12/(H12+H13))</f>
         <v/>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>299</v>
+        <v>281</v>
       </c>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
@@ -4627,9 +4319,9 @@
       <c r="H16" s="2"/>
       <c r="I16" s="2"/>
     </row>
-    <row r="17" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>300</v>
+        <v>282</v>
       </c>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
@@ -4640,9 +4332,9 @@
       <c r="H17" s="2"/>
       <c r="I17" s="2"/>
     </row>
-    <row r="18" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>301</v>
+        <v>283</v>
       </c>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
@@ -4668,103 +4360,4 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="true"/>
-  </sheetPr>
-  <dimension ref="A1:B11"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="80"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="70"/>
-  </cols>
-  <sheetData>
-    <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2"/>
-      <c r="B2" s="2"/>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="s">
-        <v>303</v>
-      </c>
-      <c r="B4" s="7" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="9" t="s">
-        <v>304</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>305</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="9" t="s">
-        <v>306</v>
-      </c>
-      <c r="B6" s="9" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="9" t="s">
-        <v>308</v>
-      </c>
-      <c r="B7" s="9" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="9" t="s">
-        <v>309</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="9" t="s">
-        <v>311</v>
-      </c>
-      <c r="B9" s="9" t="s">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="9" t="s">
-        <v>313</v>
-      </c>
-      <c r="B10" s="9" t="s">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="9" t="s">
-        <v>315</v>
-      </c>
-      <c r="B11" s="9" t="s">
-        <v>316</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A2:B2"/>
-  </mergeCells>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Worked examples: drop the cropped and the bucket-8 seasoned straight roller
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/deterioration_states/spark/stakeholder/dpd_deterioration_states_reference.xlsx
+++ b/docs/deterioration_states/spark/stakeholder/dpd_deterioration_states_reference.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="420" uniqueCount="284">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="282">
   <si>
     <t xml:space="preserve">DPD deterioration states</t>
   </si>
@@ -432,16 +432,10 @@
     <t xml:space="preserve">14 clean months, then missed every payment.</t>
   </si>
   <si>
-    <t xml:space="preserve">History starts before Jan 2024: older than a year.</t>
-  </si>
-  <si>
     <t xml:space="preserve">6 clean months, then a straight roll.</t>
   </si>
   <si>
     <t xml:space="preserve">Paid one month at 1–30 and at 31–60 DPD, still rolled.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Holding at 181–210 DPD is not Stabilized (61–180 DPD only). (6 earlier months not shown.)</t>
   </si>
   <si>
     <t xml:space="preserve">Already 121–150 DPD in the oldest month we hold.</t>
@@ -1223,7 +1217,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="63">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1405,10 +1399,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="10" fillId="14" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="17" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2416,7 +2406,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:V20"/>
+  <dimension ref="A1:V18"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
@@ -3003,41 +2993,65 @@
       <c r="V13" s="9"/>
     </row>
     <row r="14" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="14" t="s">
-        <v>35</v>
+      <c r="A14" s="15" t="s">
+        <v>39</v>
       </c>
       <c r="B14" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="C14" s="33"/>
-      <c r="D14" s="33"/>
-      <c r="E14" s="33"/>
-      <c r="F14" s="33"/>
-      <c r="G14" s="33"/>
-      <c r="H14" s="33"/>
-      <c r="I14" s="33"/>
-      <c r="J14" s="33"/>
-      <c r="K14" s="33"/>
-      <c r="L14" s="33"/>
-      <c r="M14" s="33"/>
-      <c r="N14" s="33"/>
+      <c r="C14" s="33" t="s">
+        <v>125</v>
+      </c>
+      <c r="D14" s="33" t="s">
+        <v>125</v>
+      </c>
+      <c r="E14" s="33" t="s">
+        <v>125</v>
+      </c>
+      <c r="F14" s="33" t="s">
+        <v>125</v>
+      </c>
+      <c r="G14" s="33" t="s">
+        <v>125</v>
+      </c>
+      <c r="H14" s="33" t="s">
+        <v>125</v>
+      </c>
+      <c r="I14" s="33" t="s">
+        <v>125</v>
+      </c>
+      <c r="J14" s="33" t="s">
+        <v>125</v>
+      </c>
+      <c r="K14" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" s="34" t="n">
+        <v>0</v>
+      </c>
       <c r="O14" s="34" t="n">
         <v>0</v>
       </c>
       <c r="P14" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="Q14" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="R14" s="35" t="n">
+      <c r="Q14" s="35" t="n">
         <v>2</v>
       </c>
-      <c r="S14" s="36" t="n">
+      <c r="R14" s="36" t="n">
         <v>3</v>
       </c>
-      <c r="T14" s="45" t="n">
+      <c r="S14" s="37" t="n">
         <v>4</v>
+      </c>
+      <c r="T14" s="38" t="n">
+        <v>5</v>
       </c>
       <c r="U14" s="9" t="s">
         <v>134</v>
@@ -3045,11 +3059,11 @@
       <c r="V14" s="9"/>
     </row>
     <row r="15" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="15" t="s">
-        <v>39</v>
+      <c r="A15" s="16" t="s">
+        <v>42</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="C15" s="33" t="s">
         <v>125</v>
@@ -3057,23 +3071,23 @@
       <c r="D15" s="33" t="s">
         <v>125</v>
       </c>
-      <c r="E15" s="33" t="s">
-        <v>125</v>
-      </c>
-      <c r="F15" s="33" t="s">
-        <v>125</v>
-      </c>
-      <c r="G15" s="33" t="s">
-        <v>125</v>
-      </c>
-      <c r="H15" s="33" t="s">
-        <v>125</v>
-      </c>
-      <c r="I15" s="33" t="s">
-        <v>125</v>
-      </c>
-      <c r="J15" s="33" t="s">
-        <v>125</v>
+      <c r="E15" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" s="34" t="n">
+        <v>0</v>
       </c>
       <c r="K15" s="34" t="n">
         <v>0</v>
@@ -3087,14 +3101,14 @@
       <c r="N15" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="O15" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="P15" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q15" s="35" t="n">
+      <c r="O15" s="35" t="n">
         <v>2</v>
+      </c>
+      <c r="P15" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q15" s="36" t="n">
+        <v>3</v>
       </c>
       <c r="R15" s="36" t="n">
         <v>3</v>
@@ -3111,186 +3125,54 @@
       <c r="V15" s="9"/>
     </row>
     <row r="16" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="16" t="s">
-        <v>42</v>
+      <c r="A16" s="8" t="s">
+        <v>16</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>45</v>
-      </c>
-      <c r="C16" s="33" t="s">
-        <v>125</v>
-      </c>
-      <c r="D16" s="33" t="s">
-        <v>125</v>
-      </c>
-      <c r="E16" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="G16" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="I16" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="J16" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="K16" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="L16" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="M16" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="N16" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="O16" s="35" t="n">
-        <v>2</v>
-      </c>
-      <c r="P16" s="35" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q16" s="36" t="n">
-        <v>3</v>
-      </c>
-      <c r="R16" s="36" t="n">
-        <v>3</v>
-      </c>
-      <c r="S16" s="37" t="n">
-        <v>4</v>
-      </c>
-      <c r="T16" s="38" t="n">
-        <v>5</v>
+        <v>20</v>
+      </c>
+      <c r="C16" s="33"/>
+      <c r="D16" s="33"/>
+      <c r="E16" s="33"/>
+      <c r="F16" s="33"/>
+      <c r="G16" s="33"/>
+      <c r="H16" s="33"/>
+      <c r="I16" s="33"/>
+      <c r="J16" s="33"/>
+      <c r="K16" s="33"/>
+      <c r="L16" s="33"/>
+      <c r="M16" s="33"/>
+      <c r="N16" s="33"/>
+      <c r="O16" s="40" t="n">
+        <v>6</v>
+      </c>
+      <c r="P16" s="40" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q16" s="41" t="n">
+        <v>7</v>
+      </c>
+      <c r="R16" s="41" t="n">
+        <v>7</v>
+      </c>
+      <c r="S16" s="42" t="n">
+        <v>8</v>
+      </c>
+      <c r="T16" s="44" t="n">
+        <v>9</v>
       </c>
       <c r="U16" s="9" t="s">
         <v>136</v>
       </c>
       <c r="V16" s="9"/>
     </row>
-    <row r="17" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="B17" s="10" t="s">
-        <v>38</v>
-      </c>
-      <c r="C17" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="D17" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="E17" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="F17" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="G17" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="H17" s="34" t="n">
-        <v>0</v>
-      </c>
-      <c r="I17" s="35" t="n">
-        <v>2</v>
-      </c>
-      <c r="J17" s="36" t="n">
-        <v>3</v>
-      </c>
-      <c r="K17" s="37" t="n">
-        <v>4</v>
-      </c>
-      <c r="L17" s="39" t="n">
-        <v>5</v>
-      </c>
-      <c r="M17" s="40" t="n">
-        <v>6</v>
-      </c>
-      <c r="N17" s="41" t="n">
-        <v>7</v>
-      </c>
-      <c r="O17" s="42" t="n">
-        <v>8</v>
-      </c>
-      <c r="P17" s="42" t="n">
-        <v>8</v>
-      </c>
-      <c r="Q17" s="42" t="n">
-        <v>8</v>
-      </c>
-      <c r="R17" s="42" t="n">
-        <v>8</v>
-      </c>
-      <c r="S17" s="42" t="n">
-        <v>8</v>
-      </c>
-      <c r="T17" s="46" t="n">
-        <v>8</v>
-      </c>
-      <c r="U17" s="9" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="17" t="s">
         <v>137</v>
       </c>
-      <c r="V17" s="9"/>
-    </row>
-    <row r="18" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="B18" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="C18" s="33"/>
-      <c r="D18" s="33"/>
-      <c r="E18" s="33"/>
-      <c r="F18" s="33"/>
-      <c r="G18" s="33"/>
-      <c r="H18" s="33"/>
-      <c r="I18" s="33"/>
-      <c r="J18" s="33"/>
-      <c r="K18" s="33"/>
-      <c r="L18" s="33"/>
-      <c r="M18" s="33"/>
-      <c r="N18" s="33"/>
-      <c r="O18" s="40" t="n">
-        <v>6</v>
-      </c>
-      <c r="P18" s="40" t="n">
-        <v>6</v>
-      </c>
-      <c r="Q18" s="41" t="n">
-        <v>7</v>
-      </c>
-      <c r="R18" s="41" t="n">
-        <v>7</v>
-      </c>
-      <c r="S18" s="42" t="n">
-        <v>8</v>
-      </c>
-      <c r="T18" s="44" t="n">
-        <v>9</v>
-      </c>
-      <c r="U18" s="9" t="s">
-        <v>138</v>
-      </c>
-      <c r="V18" s="9"/>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="17" t="s">
-        <v>139</v>
-      </c>
     </row>
   </sheetData>
-  <mergeCells count="23">
+  <mergeCells count="21">
     <mergeCell ref="A2:V2"/>
     <mergeCell ref="C4:D4"/>
     <mergeCell ref="E4:F4"/>
@@ -3312,8 +3194,6 @@
     <mergeCell ref="U14:V14"/>
     <mergeCell ref="U15:V15"/>
     <mergeCell ref="U16:V16"/>
-    <mergeCell ref="U17:V17"/>
-    <mergeCell ref="U18:V18"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -3341,18 +3221,18 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="C3" s="7" t="s">
         <v>141</v>
-      </c>
-      <c r="B3" s="7" t="s">
-        <v>142</v>
-      </c>
-      <c r="C3" s="7" t="s">
-        <v>143</v>
       </c>
       <c r="D3" s="7" t="s">
         <v>124</v>
@@ -3360,44 +3240,44 @@
     </row>
     <row r="4" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
+        <v>142</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>143</v>
+      </c>
+      <c r="C4" s="46" t="s">
         <v>144</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="D4" s="9" t="s">
         <v>145</v>
-      </c>
-      <c r="C4" s="47" t="s">
-        <v>146</v>
-      </c>
-      <c r="D4" s="9" t="s">
-        <v>147</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>148</v>
-      </c>
-      <c r="C5" s="47" t="s">
+        <v>146</v>
+      </c>
+      <c r="C5" s="46" t="s">
         <v>25</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
+        <v>148</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>149</v>
+      </c>
+      <c r="C6" s="46" t="s">
+        <v>34</v>
+      </c>
+      <c r="D6" s="9" t="s">
         <v>150</v>
-      </c>
-      <c r="B6" s="9" t="s">
-        <v>151</v>
-      </c>
-      <c r="C6" s="47" t="s">
-        <v>34</v>
-      </c>
-      <c r="D6" s="9" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3405,41 +3285,41 @@
         <v>26</v>
       </c>
       <c r="B7" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="C7" s="46" t="s">
+        <v>152</v>
+      </c>
+      <c r="D7" s="9" t="s">
         <v>153</v>
-      </c>
-      <c r="C7" s="47" t="s">
-        <v>154</v>
-      </c>
-      <c r="D7" s="9" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>155</v>
+      </c>
+      <c r="C8" s="46" t="s">
         <v>156</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="D8" s="9" t="s">
         <v>157</v>
-      </c>
-      <c r="C8" s="47" t="s">
-        <v>158</v>
-      </c>
-      <c r="D8" s="9" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B9" s="9" t="s">
+        <v>158</v>
+      </c>
+      <c r="C9" s="46" t="s">
+        <v>159</v>
+      </c>
+      <c r="D9" s="9" t="s">
         <v>160</v>
-      </c>
-      <c r="C9" s="47" t="s">
-        <v>161</v>
-      </c>
-      <c r="D9" s="9" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3447,13 +3327,13 @@
         <v>26</v>
       </c>
       <c r="B10" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="C10" s="46" t="s">
+        <v>162</v>
+      </c>
+      <c r="D10" s="9" t="s">
         <v>163</v>
-      </c>
-      <c r="C10" s="47" t="s">
-        <v>164</v>
-      </c>
-      <c r="D10" s="9" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3461,13 +3341,13 @@
         <v>31</v>
       </c>
       <c r="B11" s="9" t="s">
+        <v>164</v>
+      </c>
+      <c r="C11" s="46" t="s">
+        <v>165</v>
+      </c>
+      <c r="D11" s="9" t="s">
         <v>166</v>
-      </c>
-      <c r="C11" s="47" t="s">
-        <v>167</v>
-      </c>
-      <c r="D11" s="9" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3475,27 +3355,27 @@
         <v>31</v>
       </c>
       <c r="B12" s="9" t="s">
+        <v>167</v>
+      </c>
+      <c r="C12" s="46" t="s">
+        <v>168</v>
+      </c>
+      <c r="D12" s="9" t="s">
         <v>169</v>
-      </c>
-      <c r="C12" s="47" t="s">
-        <v>170</v>
-      </c>
-      <c r="D12" s="9" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="9" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="B13" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="C13" s="47" t="s">
-        <v>173</v>
+      <c r="C13" s="46" t="s">
+        <v>171</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3503,13 +3383,13 @@
         <v>92</v>
       </c>
       <c r="B14" s="9" t="s">
+        <v>173</v>
+      </c>
+      <c r="C14" s="46" t="s">
+        <v>174</v>
+      </c>
+      <c r="D14" s="9" t="s">
         <v>175</v>
-      </c>
-      <c r="C14" s="47" t="s">
-        <v>176</v>
-      </c>
-      <c r="D14" s="9" t="s">
-        <v>177</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3517,27 +3397,27 @@
         <v>92</v>
       </c>
       <c r="B15" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="C15" s="46" t="s">
+        <v>177</v>
+      </c>
+      <c r="D15" s="9" t="s">
         <v>178</v>
-      </c>
-      <c r="C15" s="47" t="s">
-        <v>179</v>
-      </c>
-      <c r="D15" s="9" t="s">
-        <v>180</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="9" t="s">
+        <v>179</v>
+      </c>
+      <c r="B16" s="9" t="s">
+        <v>180</v>
+      </c>
+      <c r="C16" s="46" t="s">
         <v>181</v>
       </c>
-      <c r="B16" s="9" t="s">
+      <c r="D16" s="9" t="s">
         <v>182</v>
-      </c>
-      <c r="C16" s="47" t="s">
-        <v>183</v>
-      </c>
-      <c r="D16" s="9" t="s">
-        <v>184</v>
       </c>
     </row>
   </sheetData>
@@ -3568,12 +3448,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -3582,41 +3462,41 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
+        <v>185</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>186</v>
+      </c>
+      <c r="C4" s="7" t="s">
         <v>187</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="D4" s="7" t="s">
         <v>188</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="E4" s="7" t="s">
         <v>189</v>
       </c>
-      <c r="D4" s="7" t="s">
+    </row>
+    <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="47" t="s">
         <v>190</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="B5" s="10" t="s">
         <v>191</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="48" t="s">
-        <v>192</v>
-      </c>
-      <c r="B5" s="10" t="s">
-        <v>193</v>
       </c>
       <c r="C5" s="10" t="s">
         <v>20</v>
       </c>
       <c r="D5" s="9" t="s">
+        <v>192</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="48" t="s">
         <v>194</v>
-      </c>
-      <c r="E5" s="9" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="49" t="s">
-        <v>196</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>30</v>
@@ -3625,15 +3505,15 @@
         <v>25</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="50" t="s">
-        <v>198</v>
+      <c r="A7" s="49" t="s">
+        <v>196</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>34</v>
@@ -3642,13 +3522,13 @@
         <v>30</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="E7" s="9"/>
     </row>
     <row r="8" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="51" t="s">
-        <v>199</v>
+      <c r="A8" s="50" t="s">
+        <v>197</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>38</v>
@@ -3657,15 +3537,15 @@
         <v>34</v>
       </c>
       <c r="D8" s="9" t="s">
+        <v>198</v>
+      </c>
+      <c r="E8" s="9" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="51" t="s">
         <v>200</v>
-      </c>
-      <c r="E8" s="9" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="52" t="s">
-        <v>202</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>45</v>
@@ -3674,79 +3554,79 @@
         <v>38</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="E9" s="9"/>
     </row>
     <row r="10" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="53" t="s">
-        <v>203</v>
+      <c r="A10" s="52" t="s">
+        <v>201</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="C10" s="10" t="s">
         <v>45</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="E10" s="9"/>
     </row>
     <row r="11" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="54" t="s">
+      <c r="A11" s="53" t="s">
+        <v>203</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>204</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>202</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>198</v>
+      </c>
+      <c r="E11" s="9" t="s">
         <v>205</v>
       </c>
-      <c r="B11" s="10" t="s">
+    </row>
+    <row r="12" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="54" t="s">
         <v>206</v>
       </c>
-      <c r="C11" s="10" t="s">
-        <v>204</v>
-      </c>
-      <c r="D11" s="9" t="s">
-        <v>200</v>
-      </c>
-      <c r="E11" s="9" t="s">
+      <c r="B12" s="10" t="s">
         <v>207</v>
       </c>
-    </row>
-    <row r="12" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="55" t="s">
+      <c r="C12" s="10" t="s">
         <v>208</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="D12" s="9" t="s">
         <v>209</v>
       </c>
-      <c r="C12" s="10" t="s">
+      <c r="E12" s="9" t="s">
         <v>210</v>
       </c>
-      <c r="D12" s="9" t="s">
+    </row>
+    <row r="13" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="55" t="s">
         <v>211</v>
       </c>
-      <c r="E12" s="9" t="s">
+      <c r="B13" s="10" t="s">
         <v>212</v>
       </c>
-    </row>
-    <row r="13" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="56" t="s">
+      <c r="C13" s="10" t="s">
+        <v>208</v>
+      </c>
+      <c r="D13" s="9" t="s">
+        <v>209</v>
+      </c>
+      <c r="E13" s="9" t="s">
         <v>213</v>
-      </c>
-      <c r="B13" s="10" t="s">
-        <v>214</v>
-      </c>
-      <c r="C13" s="10" t="s">
-        <v>210</v>
-      </c>
-      <c r="D13" s="9" t="s">
-        <v>211</v>
-      </c>
-      <c r="E13" s="9" t="s">
-        <v>215</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="B15" s="6"/>
       <c r="C15" s="6"/>
@@ -3755,21 +3635,21 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>216</v>
+      </c>
+      <c r="C16" s="7" t="s">
         <v>217</v>
-      </c>
-      <c r="B16" s="7" t="s">
-        <v>218</v>
-      </c>
-      <c r="C16" s="7" t="s">
-        <v>219</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="C17" s="10" t="s">
         <v>20</v>
@@ -3777,10 +3657,10 @@
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="9" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="C18" s="10" t="s">
         <v>25</v>
@@ -3788,35 +3668,35 @@
     </row>
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="9" t="s">
+        <v>222</v>
+      </c>
+      <c r="B19" s="9" t="s">
+        <v>223</v>
+      </c>
+      <c r="C19" s="10" t="s">
         <v>224</v>
-      </c>
-      <c r="B19" s="9" t="s">
-        <v>225</v>
-      </c>
-      <c r="C19" s="10" t="s">
-        <v>226</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="9" t="s">
+        <v>225</v>
+      </c>
+      <c r="B20" s="9" t="s">
+        <v>226</v>
+      </c>
+      <c r="C20" s="10" t="s">
         <v>227</v>
-      </c>
-      <c r="B20" s="9" t="s">
-        <v>228</v>
-      </c>
-      <c r="C20" s="10" t="s">
-        <v>229</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="9" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
     </row>
   </sheetData>
@@ -3847,157 +3727,157 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
+        <v>232</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="C4" s="7" t="s">
         <v>234</v>
       </c>
-      <c r="B4" s="7" t="s">
+    </row>
+    <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="56" t="s">
         <v>235</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="B5" s="9" t="s">
         <v>236</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="57" t="s">
+      <c r="C5" s="9" t="s">
         <v>237</v>
       </c>
-      <c r="B5" s="9" t="s">
+    </row>
+    <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="56" t="s">
         <v>238</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="B6" s="9" t="s">
         <v>239</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="57" t="s">
+      <c r="C6" s="9" t="s">
         <v>240</v>
       </c>
-      <c r="B6" s="9" t="s">
+    </row>
+    <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="56" t="s">
         <v>241</v>
       </c>
-      <c r="C6" s="9" t="s">
+      <c r="B7" s="9" t="s">
         <v>242</v>
       </c>
-    </row>
-    <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="57" t="s">
+      <c r="C7" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="B7" s="9" t="s">
+    </row>
+    <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="56" t="s">
         <v>244</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="B8" s="9" t="s">
         <v>245</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="57" t="s">
+      <c r="C8" s="9" t="s">
         <v>246</v>
       </c>
-      <c r="B8" s="9" t="s">
+    </row>
+    <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="56" t="s">
         <v>247</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="B9" s="9" t="s">
         <v>248</v>
       </c>
-    </row>
-    <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="57" t="s">
+      <c r="C9" s="9" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="56" t="s">
         <v>249</v>
       </c>
-      <c r="B9" s="9" t="s">
+      <c r="B10" s="9" t="s">
         <v>250</v>
       </c>
-      <c r="C9" s="9" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="57" t="s">
+      <c r="C10" s="9" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="56" t="s">
         <v>251</v>
       </c>
-      <c r="B10" s="9" t="s">
+      <c r="B11" s="9" t="s">
         <v>252</v>
       </c>
-      <c r="C10" s="9" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="57" t="s">
+      <c r="C11" s="9" t="s">
         <v>253</v>
       </c>
-      <c r="B11" s="9" t="s">
+    </row>
+    <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="56" t="s">
         <v>254</v>
       </c>
-      <c r="C11" s="9" t="s">
+      <c r="B12" s="9" t="s">
         <v>255</v>
       </c>
-    </row>
-    <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="57" t="s">
+      <c r="C12" s="9" t="s">
         <v>256</v>
       </c>
-      <c r="B12" s="9" t="s">
+    </row>
+    <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="56" t="s">
         <v>257</v>
       </c>
-      <c r="C12" s="9" t="s">
+      <c r="B13" s="9" t="s">
         <v>258</v>
       </c>
-    </row>
-    <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="57" t="s">
+      <c r="C13" s="9" t="s">
         <v>259</v>
       </c>
-      <c r="B13" s="9" t="s">
+    </row>
+    <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="56" t="s">
         <v>260</v>
       </c>
-      <c r="C13" s="9" t="s">
+      <c r="B14" s="9" t="s">
         <v>261</v>
       </c>
-    </row>
-    <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="57" t="s">
+      <c r="C14" s="9" t="s">
         <v>262</v>
       </c>
-      <c r="B14" s="9" t="s">
+    </row>
+    <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="56" t="s">
         <v>263</v>
       </c>
-      <c r="C14" s="9" t="s">
+      <c r="B15" s="9" t="s">
         <v>264</v>
       </c>
-    </row>
-    <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="57" t="s">
+      <c r="C15" s="9" t="s">
         <v>265</v>
       </c>
-      <c r="B15" s="9" t="s">
+    </row>
+    <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="56" t="s">
         <v>266</v>
       </c>
-      <c r="C15" s="9" t="s">
+      <c r="B16" s="9" t="s">
         <v>267</v>
       </c>
-    </row>
-    <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="57" t="s">
+      <c r="C16" s="9" t="s">
         <v>268</v>
-      </c>
-      <c r="B16" s="9" t="s">
-        <v>269</v>
-      </c>
-      <c r="C16" s="9" t="s">
-        <v>270</v>
       </c>
     </row>
   </sheetData>
@@ -4035,12 +3915,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -4056,51 +3936,51 @@
         <v>11</v>
       </c>
       <c r="B4" s="7" t="s">
+        <v>271</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>272</v>
+      </c>
+      <c r="D4" s="7" t="s">
         <v>273</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="E4" s="7" t="s">
+        <v>272</v>
+      </c>
+      <c r="F4" s="7" t="s">
         <v>274</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="G4" s="7" t="s">
+        <v>272</v>
+      </c>
+      <c r="H4" s="7" t="s">
         <v>275</v>
       </c>
-      <c r="E4" s="7" t="s">
-        <v>274</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>276</v>
-      </c>
-      <c r="G4" s="7" t="s">
-        <v>274</v>
-      </c>
-      <c r="H4" s="7" t="s">
-        <v>277</v>
-      </c>
       <c r="I4" s="7" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="B5" s="58"/>
-      <c r="C5" s="59" t="str">
+      <c r="B5" s="57"/>
+      <c r="C5" s="58" t="str">
         <f aca="false">IF($B$12=0,"",B5/$B$12)</f>
         <v/>
       </c>
-      <c r="D5" s="58"/>
-      <c r="E5" s="59" t="str">
+      <c r="D5" s="57"/>
+      <c r="E5" s="58" t="str">
         <f aca="false">IF($D$12=0,"",D5/$D$12)</f>
         <v/>
       </c>
-      <c r="F5" s="58"/>
-      <c r="G5" s="59" t="str">
+      <c r="F5" s="57"/>
+      <c r="G5" s="58" t="str">
         <f aca="false">IF($F$12=0,"",F5/$F$12)</f>
         <v/>
       </c>
-      <c r="H5" s="58"/>
-      <c r="I5" s="59" t="str">
+      <c r="H5" s="57"/>
+      <c r="I5" s="58" t="str">
         <f aca="false">IF($H$12=0,"",H5/$H$12)</f>
         <v/>
       </c>
@@ -4109,23 +3989,23 @@
       <c r="A6" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="B6" s="58"/>
-      <c r="C6" s="59" t="str">
+      <c r="B6" s="57"/>
+      <c r="C6" s="58" t="str">
         <f aca="false">IF($B$12=0,"",B6/$B$12)</f>
         <v/>
       </c>
-      <c r="D6" s="58"/>
-      <c r="E6" s="59" t="str">
+      <c r="D6" s="57"/>
+      <c r="E6" s="58" t="str">
         <f aca="false">IF($D$12=0,"",D6/$D$12)</f>
         <v/>
       </c>
-      <c r="F6" s="58"/>
-      <c r="G6" s="59" t="str">
+      <c r="F6" s="57"/>
+      <c r="G6" s="58" t="str">
         <f aca="false">IF($F$12=0,"",F6/$F$12)</f>
         <v/>
       </c>
-      <c r="H6" s="58"/>
-      <c r="I6" s="59" t="str">
+      <c r="H6" s="57"/>
+      <c r="I6" s="58" t="str">
         <f aca="false">IF($H$12=0,"",H6/$H$12)</f>
         <v/>
       </c>
@@ -4134,23 +4014,23 @@
       <c r="A7" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="B7" s="58"/>
-      <c r="C7" s="59" t="str">
+      <c r="B7" s="57"/>
+      <c r="C7" s="58" t="str">
         <f aca="false">IF($B$12=0,"",B7/$B$12)</f>
         <v/>
       </c>
-      <c r="D7" s="58"/>
-      <c r="E7" s="59" t="str">
+      <c r="D7" s="57"/>
+      <c r="E7" s="58" t="str">
         <f aca="false">IF($D$12=0,"",D7/$D$12)</f>
         <v/>
       </c>
-      <c r="F7" s="58"/>
-      <c r="G7" s="59" t="str">
+      <c r="F7" s="57"/>
+      <c r="G7" s="58" t="str">
         <f aca="false">IF($F$12=0,"",F7/$F$12)</f>
         <v/>
       </c>
-      <c r="H7" s="58"/>
-      <c r="I7" s="59" t="str">
+      <c r="H7" s="57"/>
+      <c r="I7" s="58" t="str">
         <f aca="false">IF($H$12=0,"",H7/$H$12)</f>
         <v/>
       </c>
@@ -4159,23 +4039,23 @@
       <c r="A8" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="B8" s="58"/>
-      <c r="C8" s="59" t="str">
+      <c r="B8" s="57"/>
+      <c r="C8" s="58" t="str">
         <f aca="false">IF($B$12=0,"",B8/$B$12)</f>
         <v/>
       </c>
-      <c r="D8" s="58"/>
-      <c r="E8" s="59" t="str">
+      <c r="D8" s="57"/>
+      <c r="E8" s="58" t="str">
         <f aca="false">IF($D$12=0,"",D8/$D$12)</f>
         <v/>
       </c>
-      <c r="F8" s="58"/>
-      <c r="G8" s="59" t="str">
+      <c r="F8" s="57"/>
+      <c r="G8" s="58" t="str">
         <f aca="false">IF($F$12=0,"",F8/$F$12)</f>
         <v/>
       </c>
-      <c r="H8" s="58"/>
-      <c r="I8" s="59" t="str">
+      <c r="H8" s="57"/>
+      <c r="I8" s="58" t="str">
         <f aca="false">IF($H$12=0,"",H8/$H$12)</f>
         <v/>
       </c>
@@ -4184,23 +4064,23 @@
       <c r="A9" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="B9" s="58"/>
-      <c r="C9" s="59" t="str">
+      <c r="B9" s="57"/>
+      <c r="C9" s="58" t="str">
         <f aca="false">IF($B$12=0,"",B9/$B$12)</f>
         <v/>
       </c>
-      <c r="D9" s="58"/>
-      <c r="E9" s="59" t="str">
+      <c r="D9" s="57"/>
+      <c r="E9" s="58" t="str">
         <f aca="false">IF($D$12=0,"",D9/$D$12)</f>
         <v/>
       </c>
-      <c r="F9" s="58"/>
-      <c r="G9" s="59" t="str">
+      <c r="F9" s="57"/>
+      <c r="G9" s="58" t="str">
         <f aca="false">IF($F$12=0,"",F9/$F$12)</f>
         <v/>
       </c>
-      <c r="H9" s="58"/>
-      <c r="I9" s="59" t="str">
+      <c r="H9" s="57"/>
+      <c r="I9" s="58" t="str">
         <f aca="false">IF($H$12=0,"",H9/$H$12)</f>
         <v/>
       </c>
@@ -4209,23 +4089,23 @@
       <c r="A10" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="B10" s="58"/>
-      <c r="C10" s="59" t="str">
+      <c r="B10" s="57"/>
+      <c r="C10" s="58" t="str">
         <f aca="false">IF($B$12=0,"",B10/$B$12)</f>
         <v/>
       </c>
-      <c r="D10" s="58"/>
-      <c r="E10" s="59" t="str">
+      <c r="D10" s="57"/>
+      <c r="E10" s="58" t="str">
         <f aca="false">IF($D$12=0,"",D10/$D$12)</f>
         <v/>
       </c>
-      <c r="F10" s="58"/>
-      <c r="G10" s="59" t="str">
+      <c r="F10" s="57"/>
+      <c r="G10" s="58" t="str">
         <f aca="false">IF($F$12=0,"",F10/$F$12)</f>
         <v/>
       </c>
-      <c r="H10" s="58"/>
-      <c r="I10" s="59" t="str">
+      <c r="H10" s="57"/>
+      <c r="I10" s="58" t="str">
         <f aca="false">IF($H$12=0,"",H10/$H$12)</f>
         <v/>
       </c>
@@ -4234,81 +4114,81 @@
       <c r="A11" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="B11" s="58"/>
-      <c r="C11" s="59" t="str">
+      <c r="B11" s="57"/>
+      <c r="C11" s="58" t="str">
         <f aca="false">IF($B$12=0,"",B11/$B$12)</f>
         <v/>
       </c>
-      <c r="D11" s="58"/>
-      <c r="E11" s="59" t="str">
+      <c r="D11" s="57"/>
+      <c r="E11" s="58" t="str">
         <f aca="false">IF($D$12=0,"",D11/$D$12)</f>
         <v/>
       </c>
-      <c r="F11" s="58"/>
-      <c r="G11" s="59" t="str">
+      <c r="F11" s="57"/>
+      <c r="G11" s="58" t="str">
         <f aca="false">IF($F$12=0,"",F11/$F$12)</f>
         <v/>
       </c>
-      <c r="H11" s="58"/>
-      <c r="I11" s="59" t="str">
+      <c r="H11" s="57"/>
+      <c r="I11" s="58" t="str">
         <f aca="false">IF($H$12=0,"",H11/$H$12)</f>
         <v/>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="23" t="s">
-        <v>278</v>
-      </c>
-      <c r="B12" s="60" t="n">
+        <v>276</v>
+      </c>
+      <c r="B12" s="59" t="n">
         <f aca="false">SUM(B5:B11)</f>
         <v>0</v>
       </c>
-      <c r="D12" s="60" t="n">
+      <c r="D12" s="59" t="n">
         <f aca="false">SUM(D5:D11)</f>
         <v>0</v>
       </c>
-      <c r="F12" s="60" t="n">
+      <c r="F12" s="59" t="n">
         <f aca="false">SUM(F5:F11)</f>
         <v>0</v>
       </c>
-      <c r="H12" s="60" t="n">
+      <c r="H12" s="59" t="n">
         <f aca="false">SUM(H5:H11)</f>
         <v>0</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="61" t="s">
-        <v>279</v>
-      </c>
-      <c r="B13" s="62"/>
-      <c r="D13" s="62"/>
-      <c r="F13" s="62"/>
-      <c r="H13" s="62"/>
+      <c r="A13" s="60" t="s">
+        <v>277</v>
+      </c>
+      <c r="B13" s="61"/>
+      <c r="D13" s="61"/>
+      <c r="F13" s="61"/>
+      <c r="H13" s="61"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="23" t="s">
-        <v>280</v>
-      </c>
-      <c r="B14" s="63" t="str">
+        <v>278</v>
+      </c>
+      <c r="B14" s="62" t="str">
         <f aca="false">IF((B12+B13)=0,"",B12/(B12+B13))</f>
         <v/>
       </c>
-      <c r="D14" s="63" t="str">
+      <c r="D14" s="62" t="str">
         <f aca="false">IF((D12+D13)=0,"",D12/(D12+D13))</f>
         <v/>
       </c>
-      <c r="F14" s="63" t="str">
+      <c r="F14" s="62" t="str">
         <f aca="false">IF((F12+F13)=0,"",F12/(F12+F13))</f>
         <v/>
       </c>
-      <c r="H14" s="63" t="str">
+      <c r="H14" s="62" t="str">
         <f aca="false">IF((H12+H13)=0,"",H12/(H12+H13))</f>
         <v/>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
@@ -4321,7 +4201,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
@@ -4334,7 +4214,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>

</xml_diff>

<commit_message>
Worked examples: blank cells before the history starts; drop the footnote
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/deterioration_states/spark/stakeholder/dpd_deterioration_states_reference.xlsx
+++ b/docs/deterioration_states/spark/stakeholder/dpd_deterioration_states_reference.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="282">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="280">
   <si>
     <t xml:space="preserve">DPD deterioration states</t>
   </si>
@@ -405,9 +405,6 @@
     <t xml:space="preserve">Why</t>
   </si>
   <si>
-    <t xml:space="preserve">·</t>
-  </si>
-  <si>
     <t xml:space="preserve">3 clean months, then one bucket worse every month.</t>
   </si>
   <si>
@@ -439,9 +436,6 @@
   </si>
   <si>
     <t xml:space="preserve">Already 121–150 DPD in the oldest month we hold.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">'·' = no history yet (account not open).</t>
   </si>
   <si>
     <t xml:space="preserve">Thresholds</t>
@@ -890,7 +884,7 @@
     <numFmt numFmtId="166" formatCode="0.0%"/>
     <numFmt numFmtId="167" formatCode="0.00%"/>
   </numFmts>
-  <fonts count="20">
+  <fonts count="19">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1001,13 +995,6 @@
       <b val="true"/>
       <sz val="8"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FFBFBFBF"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -1350,23 +1337,23 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="11" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="11" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="12" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="12" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="13" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="13" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="14" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="14" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1374,23 +1361,23 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="15" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="15" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="16" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="16" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="6" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="17" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="17" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="18" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="18" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1446,7 +1433,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="19" fillId="19" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="18" fillId="19" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1462,7 +1449,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="19" fillId="19" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="18" fillId="19" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2406,7 +2393,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:V18"/>
+  <dimension ref="A1:V16"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="28"/>
@@ -2561,39 +2548,17 @@
       <c r="B7" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="C7" s="33" t="s">
-        <v>125</v>
-      </c>
-      <c r="D7" s="33" t="s">
-        <v>125</v>
-      </c>
-      <c r="E7" s="33" t="s">
-        <v>125</v>
-      </c>
-      <c r="F7" s="33" t="s">
-        <v>125</v>
-      </c>
-      <c r="G7" s="33" t="s">
-        <v>125</v>
-      </c>
-      <c r="H7" s="33" t="s">
-        <v>125</v>
-      </c>
-      <c r="I7" s="33" t="s">
-        <v>125</v>
-      </c>
-      <c r="J7" s="33" t="s">
-        <v>125</v>
-      </c>
-      <c r="K7" s="33" t="s">
-        <v>125</v>
-      </c>
-      <c r="L7" s="33" t="s">
-        <v>125</v>
-      </c>
-      <c r="M7" s="33" t="s">
-        <v>125</v>
-      </c>
+      <c r="C7" s="33"/>
+      <c r="D7" s="33"/>
+      <c r="E7" s="33"/>
+      <c r="F7" s="33"/>
+      <c r="G7" s="33"/>
+      <c r="H7" s="33"/>
+      <c r="I7" s="33"/>
+      <c r="J7" s="33"/>
+      <c r="K7" s="33"/>
+      <c r="L7" s="33"/>
+      <c r="M7" s="33"/>
       <c r="N7" s="34" t="n">
         <v>0</v>
       </c>
@@ -2616,7 +2581,7 @@
         <v>5</v>
       </c>
       <c r="U7" s="9" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="V7" s="9"/>
     </row>
@@ -2627,27 +2592,13 @@
       <c r="B8" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="C8" s="33" t="s">
-        <v>125</v>
-      </c>
-      <c r="D8" s="33" t="s">
-        <v>125</v>
-      </c>
-      <c r="E8" s="33" t="s">
-        <v>125</v>
-      </c>
-      <c r="F8" s="33" t="s">
-        <v>125</v>
-      </c>
-      <c r="G8" s="33" t="s">
-        <v>125</v>
-      </c>
-      <c r="H8" s="33" t="s">
-        <v>125</v>
-      </c>
-      <c r="I8" s="33" t="s">
-        <v>125</v>
-      </c>
+      <c r="C8" s="33"/>
+      <c r="D8" s="33"/>
+      <c r="E8" s="33"/>
+      <c r="F8" s="33"/>
+      <c r="G8" s="33"/>
+      <c r="H8" s="33"/>
+      <c r="I8" s="33"/>
       <c r="J8" s="34" t="n">
         <v>0</v>
       </c>
@@ -2682,7 +2633,7 @@
         <v>9</v>
       </c>
       <c r="U8" s="9" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="V8" s="9"/>
     </row>
@@ -2693,9 +2644,7 @@
       <c r="B9" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="C9" s="33" t="s">
-        <v>125</v>
-      </c>
+      <c r="C9" s="33"/>
       <c r="D9" s="34" t="n">
         <v>0</v>
       </c>
@@ -2748,7 +2697,7 @@
         <v>5</v>
       </c>
       <c r="U9" s="9" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="V9" s="9"/>
     </row>
@@ -2814,7 +2763,7 @@
         <v>4</v>
       </c>
       <c r="U10" s="9" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="V10" s="9"/>
     </row>
@@ -2823,7 +2772,7 @@
         <v>26</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C11" s="33"/>
       <c r="D11" s="33"/>
@@ -2856,7 +2805,7 @@
         <v>5</v>
       </c>
       <c r="U11" s="9" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="V11" s="9"/>
     </row>
@@ -2867,12 +2816,8 @@
       <c r="B12" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="C12" s="33" t="s">
-        <v>125</v>
-      </c>
-      <c r="D12" s="33" t="s">
-        <v>125</v>
-      </c>
+      <c r="C12" s="33"/>
+      <c r="D12" s="33"/>
       <c r="E12" s="34" t="n">
         <v>0</v>
       </c>
@@ -2922,7 +2867,7 @@
         <v>5</v>
       </c>
       <c r="U12" s="9" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="V12" s="9"/>
     </row>
@@ -2988,7 +2933,7 @@
         <v>5</v>
       </c>
       <c r="U13" s="9" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="V13" s="9"/>
     </row>
@@ -2999,30 +2944,14 @@
       <c r="B14" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="C14" s="33" t="s">
-        <v>125</v>
-      </c>
-      <c r="D14" s="33" t="s">
-        <v>125</v>
-      </c>
-      <c r="E14" s="33" t="s">
-        <v>125</v>
-      </c>
-      <c r="F14" s="33" t="s">
-        <v>125</v>
-      </c>
-      <c r="G14" s="33" t="s">
-        <v>125</v>
-      </c>
-      <c r="H14" s="33" t="s">
-        <v>125</v>
-      </c>
-      <c r="I14" s="33" t="s">
-        <v>125</v>
-      </c>
-      <c r="J14" s="33" t="s">
-        <v>125</v>
-      </c>
+      <c r="C14" s="33"/>
+      <c r="D14" s="33"/>
+      <c r="E14" s="33"/>
+      <c r="F14" s="33"/>
+      <c r="G14" s="33"/>
+      <c r="H14" s="33"/>
+      <c r="I14" s="33"/>
+      <c r="J14" s="33"/>
       <c r="K14" s="34" t="n">
         <v>0</v>
       </c>
@@ -3054,7 +2983,7 @@
         <v>5</v>
       </c>
       <c r="U14" s="9" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="V14" s="9"/>
     </row>
@@ -3065,12 +2994,8 @@
       <c r="B15" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="C15" s="33" t="s">
-        <v>125</v>
-      </c>
-      <c r="D15" s="33" t="s">
-        <v>125</v>
-      </c>
+      <c r="C15" s="33"/>
+      <c r="D15" s="33"/>
       <c r="E15" s="34" t="n">
         <v>0</v>
       </c>
@@ -3120,7 +3045,7 @@
         <v>5</v>
       </c>
       <c r="U15" s="9" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="V15" s="9"/>
     </row>
@@ -3162,14 +3087,9 @@
         <v>9</v>
       </c>
       <c r="U16" s="9" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="V16" s="9"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="17" t="s">
-        <v>137</v>
-      </c>
     </row>
   </sheetData>
   <mergeCells count="21">
@@ -3221,18 +3141,18 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="C3" s="7" t="s">
         <v>139</v>
-      </c>
-      <c r="B3" s="7" t="s">
-        <v>140</v>
-      </c>
-      <c r="C3" s="7" t="s">
-        <v>141</v>
       </c>
       <c r="D3" s="7" t="s">
         <v>124</v>
@@ -3240,44 +3160,44 @@
     </row>
     <row r="4" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>141</v>
+      </c>
+      <c r="C4" s="46" t="s">
         <v>142</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="D4" s="9" t="s">
         <v>143</v>
-      </c>
-      <c r="C4" s="46" t="s">
-        <v>144</v>
-      </c>
-      <c r="D4" s="9" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="C5" s="46" t="s">
         <v>25</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C6" s="46" t="s">
         <v>34</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3285,41 +3205,41 @@
         <v>26</v>
       </c>
       <c r="B7" s="9" t="s">
+        <v>149</v>
+      </c>
+      <c r="C7" s="46" t="s">
+        <v>150</v>
+      </c>
+      <c r="D7" s="9" t="s">
         <v>151</v>
-      </c>
-      <c r="C7" s="46" t="s">
-        <v>152</v>
-      </c>
-      <c r="D7" s="9" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="9" t="s">
+        <v>152</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="C8" s="46" t="s">
         <v>154</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="D8" s="9" t="s">
         <v>155</v>
-      </c>
-      <c r="C8" s="46" t="s">
-        <v>156</v>
-      </c>
-      <c r="D8" s="9" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="B9" s="9" t="s">
+        <v>156</v>
+      </c>
+      <c r="C9" s="46" t="s">
+        <v>157</v>
+      </c>
+      <c r="D9" s="9" t="s">
         <v>158</v>
-      </c>
-      <c r="C9" s="46" t="s">
-        <v>159</v>
-      </c>
-      <c r="D9" s="9" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3327,13 +3247,13 @@
         <v>26</v>
       </c>
       <c r="B10" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="C10" s="46" t="s">
+        <v>160</v>
+      </c>
+      <c r="D10" s="9" t="s">
         <v>161</v>
-      </c>
-      <c r="C10" s="46" t="s">
-        <v>162</v>
-      </c>
-      <c r="D10" s="9" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3341,13 +3261,13 @@
         <v>31</v>
       </c>
       <c r="B11" s="9" t="s">
+        <v>162</v>
+      </c>
+      <c r="C11" s="46" t="s">
+        <v>163</v>
+      </c>
+      <c r="D11" s="9" t="s">
         <v>164</v>
-      </c>
-      <c r="C11" s="46" t="s">
-        <v>165</v>
-      </c>
-      <c r="D11" s="9" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3355,27 +3275,27 @@
         <v>31</v>
       </c>
       <c r="B12" s="9" t="s">
+        <v>165</v>
+      </c>
+      <c r="C12" s="46" t="s">
+        <v>166</v>
+      </c>
+      <c r="D12" s="9" t="s">
         <v>167</v>
-      </c>
-      <c r="C12" s="46" t="s">
-        <v>168</v>
-      </c>
-      <c r="D12" s="9" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="9" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B13" s="9" t="s">
         <v>88</v>
       </c>
       <c r="C13" s="46" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3383,13 +3303,13 @@
         <v>92</v>
       </c>
       <c r="B14" s="9" t="s">
+        <v>171</v>
+      </c>
+      <c r="C14" s="46" t="s">
+        <v>172</v>
+      </c>
+      <c r="D14" s="9" t="s">
         <v>173</v>
-      </c>
-      <c r="C14" s="46" t="s">
-        <v>174</v>
-      </c>
-      <c r="D14" s="9" t="s">
-        <v>175</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3397,27 +3317,27 @@
         <v>92</v>
       </c>
       <c r="B15" s="9" t="s">
+        <v>174</v>
+      </c>
+      <c r="C15" s="46" t="s">
+        <v>175</v>
+      </c>
+      <c r="D15" s="9" t="s">
         <v>176</v>
-      </c>
-      <c r="C15" s="46" t="s">
-        <v>177</v>
-      </c>
-      <c r="D15" s="9" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="9" t="s">
+        <v>177</v>
+      </c>
+      <c r="B16" s="9" t="s">
+        <v>178</v>
+      </c>
+      <c r="C16" s="46" t="s">
         <v>179</v>
       </c>
-      <c r="B16" s="9" t="s">
+      <c r="D16" s="9" t="s">
         <v>180</v>
-      </c>
-      <c r="C16" s="46" t="s">
-        <v>181</v>
-      </c>
-      <c r="D16" s="9" t="s">
-        <v>182</v>
       </c>
     </row>
   </sheetData>
@@ -3448,12 +3368,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -3462,41 +3382,41 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
+        <v>183</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="C4" s="7" t="s">
         <v>185</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="D4" s="7" t="s">
         <v>186</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="E4" s="7" t="s">
         <v>187</v>
-      </c>
-      <c r="D4" s="7" t="s">
-        <v>188</v>
-      </c>
-      <c r="E4" s="7" t="s">
-        <v>189</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="47" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="C5" s="10" t="s">
         <v>20</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="48" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="B6" s="10" t="s">
         <v>30</v>
@@ -3505,15 +3425,15 @@
         <v>25</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="49" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>34</v>
@@ -3522,13 +3442,13 @@
         <v>30</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="E7" s="9"/>
     </row>
     <row r="8" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="50" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="B8" s="10" t="s">
         <v>38</v>
@@ -3537,15 +3457,15 @@
         <v>34</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="51" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="B9" s="10" t="s">
         <v>45</v>
@@ -3554,79 +3474,79 @@
         <v>38</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="E9" s="9"/>
     </row>
     <row r="10" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="52" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="C10" s="10" t="s">
         <v>45</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="E10" s="9"/>
     </row>
     <row r="11" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="53" t="s">
+        <v>201</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>202</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>200</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>196</v>
+      </c>
+      <c r="E11" s="9" t="s">
         <v>203</v>
-      </c>
-      <c r="B11" s="10" t="s">
-        <v>204</v>
-      </c>
-      <c r="C11" s="10" t="s">
-        <v>202</v>
-      </c>
-      <c r="D11" s="9" t="s">
-        <v>198</v>
-      </c>
-      <c r="E11" s="9" t="s">
-        <v>205</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="54" t="s">
+        <v>204</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>205</v>
+      </c>
+      <c r="C12" s="10" t="s">
         <v>206</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="D12" s="9" t="s">
         <v>207</v>
       </c>
-      <c r="C12" s="10" t="s">
+      <c r="E12" s="9" t="s">
         <v>208</v>
-      </c>
-      <c r="D12" s="9" t="s">
-        <v>209</v>
-      </c>
-      <c r="E12" s="9" t="s">
-        <v>210</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="55" t="s">
+        <v>209</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>210</v>
+      </c>
+      <c r="C13" s="10" t="s">
+        <v>206</v>
+      </c>
+      <c r="D13" s="9" t="s">
+        <v>207</v>
+      </c>
+      <c r="E13" s="9" t="s">
         <v>211</v>
-      </c>
-      <c r="B13" s="10" t="s">
-        <v>212</v>
-      </c>
-      <c r="C13" s="10" t="s">
-        <v>208</v>
-      </c>
-      <c r="D13" s="9" t="s">
-        <v>209</v>
-      </c>
-      <c r="E13" s="9" t="s">
-        <v>213</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="B15" s="6"/>
       <c r="C15" s="6"/>
@@ -3635,21 +3555,21 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
+        <v>213</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>214</v>
+      </c>
+      <c r="C16" s="7" t="s">
         <v>215</v>
-      </c>
-      <c r="B16" s="7" t="s">
-        <v>216</v>
-      </c>
-      <c r="C16" s="7" t="s">
-        <v>217</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="C17" s="10" t="s">
         <v>20</v>
@@ -3657,10 +3577,10 @@
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="9" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="C18" s="10" t="s">
         <v>25</v>
@@ -3668,35 +3588,35 @@
     </row>
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="9" t="s">
+        <v>220</v>
+      </c>
+      <c r="B19" s="9" t="s">
+        <v>221</v>
+      </c>
+      <c r="C19" s="10" t="s">
         <v>222</v>
-      </c>
-      <c r="B19" s="9" t="s">
-        <v>223</v>
-      </c>
-      <c r="C19" s="10" t="s">
-        <v>224</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="9" t="s">
+        <v>223</v>
+      </c>
+      <c r="B20" s="9" t="s">
+        <v>224</v>
+      </c>
+      <c r="C20" s="10" t="s">
         <v>225</v>
-      </c>
-      <c r="B20" s="9" t="s">
-        <v>226</v>
-      </c>
-      <c r="C20" s="10" t="s">
-        <v>227</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="9" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
     </row>
   </sheetData>
@@ -3727,157 +3647,157 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
+        <v>230</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>231</v>
+      </c>
+      <c r="C4" s="7" t="s">
         <v>232</v>
-      </c>
-      <c r="B4" s="7" t="s">
-        <v>233</v>
-      </c>
-      <c r="C4" s="7" t="s">
-        <v>234</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="56" t="s">
+        <v>233</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="C5" s="9" t="s">
         <v>235</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>236</v>
-      </c>
-      <c r="C5" s="9" t="s">
-        <v>237</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="56" t="s">
+        <v>236</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>237</v>
+      </c>
+      <c r="C6" s="9" t="s">
         <v>238</v>
-      </c>
-      <c r="B6" s="9" t="s">
-        <v>239</v>
-      </c>
-      <c r="C6" s="9" t="s">
-        <v>240</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="56" t="s">
+        <v>239</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>240</v>
+      </c>
+      <c r="C7" s="9" t="s">
         <v>241</v>
-      </c>
-      <c r="B7" s="9" t="s">
-        <v>242</v>
-      </c>
-      <c r="C7" s="9" t="s">
-        <v>243</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="56" t="s">
+        <v>242</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>243</v>
+      </c>
+      <c r="C8" s="9" t="s">
         <v>244</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>245</v>
-      </c>
-      <c r="C8" s="9" t="s">
-        <v>246</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="56" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="56" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="56" t="s">
+        <v>249</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>250</v>
+      </c>
+      <c r="C11" s="9" t="s">
         <v>251</v>
-      </c>
-      <c r="B11" s="9" t="s">
-        <v>252</v>
-      </c>
-      <c r="C11" s="9" t="s">
-        <v>253</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="56" t="s">
+        <v>252</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>253</v>
+      </c>
+      <c r="C12" s="9" t="s">
         <v>254</v>
-      </c>
-      <c r="B12" s="9" t="s">
-        <v>255</v>
-      </c>
-      <c r="C12" s="9" t="s">
-        <v>256</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="56" t="s">
+        <v>255</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>256</v>
+      </c>
+      <c r="C13" s="9" t="s">
         <v>257</v>
-      </c>
-      <c r="B13" s="9" t="s">
-        <v>258</v>
-      </c>
-      <c r="C13" s="9" t="s">
-        <v>259</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="56" t="s">
+        <v>258</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>259</v>
+      </c>
+      <c r="C14" s="9" t="s">
         <v>260</v>
-      </c>
-      <c r="B14" s="9" t="s">
-        <v>261</v>
-      </c>
-      <c r="C14" s="9" t="s">
-        <v>262</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="56" t="s">
+        <v>261</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>262</v>
+      </c>
+      <c r="C15" s="9" t="s">
         <v>263</v>
-      </c>
-      <c r="B15" s="9" t="s">
-        <v>264</v>
-      </c>
-      <c r="C15" s="9" t="s">
-        <v>265</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="56" t="s">
+        <v>264</v>
+      </c>
+      <c r="B16" s="9" t="s">
+        <v>265</v>
+      </c>
+      <c r="C16" s="9" t="s">
         <v>266</v>
-      </c>
-      <c r="B16" s="9" t="s">
-        <v>267</v>
-      </c>
-      <c r="C16" s="9" t="s">
-        <v>268</v>
       </c>
     </row>
   </sheetData>
@@ -3915,12 +3835,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -3936,28 +3856,28 @@
         <v>11</v>
       </c>
       <c r="B4" s="7" t="s">
+        <v>269</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>270</v>
+      </c>
+      <c r="D4" s="7" t="s">
         <v>271</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="E4" s="7" t="s">
+        <v>270</v>
+      </c>
+      <c r="F4" s="7" t="s">
         <v>272</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="G4" s="7" t="s">
+        <v>270</v>
+      </c>
+      <c r="H4" s="7" t="s">
         <v>273</v>
       </c>
-      <c r="E4" s="7" t="s">
-        <v>272</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>274</v>
-      </c>
-      <c r="G4" s="7" t="s">
-        <v>272</v>
-      </c>
-      <c r="H4" s="7" t="s">
-        <v>275</v>
-      </c>
       <c r="I4" s="7" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4137,7 +4057,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="23" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="B12" s="59" t="n">
         <f aca="false">SUM(B5:B11)</f>
@@ -4158,7 +4078,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="60" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="B13" s="61"/>
       <c r="D13" s="61"/>
@@ -4167,7 +4087,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="23" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="B14" s="62" t="str">
         <f aca="false">IF((B12+B13)=0,"",B12/(B12+B13))</f>
@@ -4188,7 +4108,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
@@ -4201,7 +4121,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
@@ -4214,7 +4134,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>

</xml_diff>

<commit_message>
Thresholds: clearer slip and straight-roll wording; one term for short slips
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/deterioration_states/spark/stakeholder/dpd_deterioration_states_reference.xlsx
+++ b/docs/deterioration_states/spark/stakeholder/dpd_deterioration_states_reference.xlsx
@@ -462,19 +462,19 @@
     <t xml:space="preserve">Someone who never pays misses the 1st or 2nd bill.</t>
   </si>
   <si>
-    <t xml:space="preserve">Short paid-off slips allowed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">One brief slip doesn't show good behaviour.</t>
+    <t xml:space="preserve">Earlier short slips allowed (1–2 months, paid off)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One quickly repaid late payment does not rule out EPD.</t>
   </si>
   <si>
     <t xml:space="preserve">Straight roller</t>
   </si>
   <si>
-    <t xml:space="preserve">Months from first miss to 61–90 DPD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Three misses in a row: nothing paid on the way.</t>
+    <t xml:space="preserve">Delinquent months to reach 61–90 DPD (1–30, 31–60, 61–90)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One bucket a month: nothing paid on the way.</t>
   </si>
   <si>
     <t xml:space="preserve">Last 6 months within one bucket of today's</t>
@@ -483,7 +483,7 @@
     <t xml:space="preserve">5 of 6</t>
   </si>
   <si>
-    <t xml:space="preserve">The bank's existing rule.</t>
+    <t xml:space="preserve">Staying near the same bucket means about one month's due is paid each month.</t>
   </si>
   <si>
     <t xml:space="preserve">Stabilized (long-term)</t>
@@ -795,7 +795,7 @@
     <t xml:space="preserve">As for history before the window start.</t>
   </si>
   <si>
-    <t xml:space="preserve">One-month blips (4 0 4, 0 3 0)</t>
+    <t xml:space="preserve">One-month data errors (4 0 4, 0 3 0)</t>
   </si>
   <si>
     <t xml:space="preserve">Corrected to the neighbours.</t>

</xml_diff>

<commit_message>
Thresholds: reasons stated on their own merits, no appeals to bank or common practice
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/deterioration_states/spark/stakeholder/dpd_deterioration_states_reference.xlsx
+++ b/docs/deterioration_states/spark/stakeholder/dpd_deterioration_states_reference.xlsx
@@ -522,7 +522,7 @@
     <t xml:space="preserve">31+ DPD</t>
   </si>
   <si>
-    <t xml:space="preserve">Matches the bank's re-default view.</t>
+    <t xml:space="preserve">A cure from 31+ DPD shows real ability to catch up.</t>
   </si>
   <si>
     <t xml:space="preserve">Months since it ended</t>
@@ -531,7 +531,7 @@
     <t xml:space="preserve">≤ 12</t>
   </si>
   <si>
-    <t xml:space="preserve">Common re-default window.</t>
+    <t xml:space="preserve">A relapse within a year points to the same underlying problem.</t>
   </si>
   <si>
     <t xml:space="preserve">Seasoned vs early-life</t>
@@ -540,7 +540,7 @@
     <t xml:space="preserve">12+</t>
   </si>
   <si>
-    <t xml:space="preserve">Standard first-year window.</t>
+    <t xml:space="preserve">First-year defaults point to acquisition; later ones to a change in circumstances.</t>
   </si>
   <si>
     <t xml:space="preserve">CC data used from</t>

</xml_diff>

<commit_message>
Data handling: drop the RL first-month and CC cycle-shift rows
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/deterioration_states/spark/stakeholder/dpd_deterioration_states_reference.xlsx
+++ b/docs/deterioration_states/spark/stakeholder/dpd_deterioration_states_reference.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="280">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="275">
   <si>
     <t xml:space="preserve">DPD deterioration states</t>
   </si>
@@ -747,28 +747,13 @@
     <t xml:space="preserve">Unknown, unless Stabilized.</t>
   </si>
   <si>
-    <t xml:space="preserve">RL loan 1–30 DPD in its first month</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Normal: its first payment is due that month.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Classified as usual.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Two bills in one month, none in the next (CC)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">One bill moved to the empty month.</t>
+    <t xml:space="preserve">Missing month between two equal buckets</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Filled with that bucket.</t>
   </si>
   <si>
     <t xml:space="preserve">None.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Missing month between two equal buckets</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Filled with that bucket.</t>
   </si>
   <si>
     <t xml:space="preserve">Missing month where only a straight roll fits</t>
@@ -3638,7 +3623,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
@@ -3709,18 +3694,18 @@
         <v>243</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="56" t="s">
+        <v>244</v>
+      </c>
+      <c r="B9" s="9" t="s">
         <v>245</v>
       </c>
-      <c r="B9" s="9" t="s">
+      <c r="C9" s="9" t="s">
         <v>246</v>
-      </c>
-      <c r="C9" s="9" t="s">
-        <v>244</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3731,73 +3716,51 @@
         <v>248</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="56" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="56" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="56" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="56" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="56" t="s">
         <v>261</v>
-      </c>
-      <c r="B15" s="9" t="s">
-        <v>262</v>
-      </c>
-      <c r="C15" s="9" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="56" t="s">
-        <v>264</v>
-      </c>
-      <c r="B16" s="9" t="s">
-        <v>265</v>
-      </c>
-      <c r="C16" s="9" t="s">
-        <v>266</v>
       </c>
     </row>
   </sheetData>
@@ -3835,12 +3798,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -3856,28 +3819,28 @@
         <v>11</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>271</v>
+        <v>266</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>272</v>
+        <v>267</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="I4" s="7" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4057,7 +4020,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="23" t="s">
-        <v>274</v>
+        <v>269</v>
       </c>
       <c r="B12" s="59" t="n">
         <f aca="false">SUM(B5:B11)</f>
@@ -4078,7 +4041,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="60" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="B13" s="61"/>
       <c r="D13" s="61"/>
@@ -4087,7 +4050,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="23" t="s">
-        <v>276</v>
+        <v>271</v>
       </c>
       <c r="B14" s="62" t="str">
         <f aca="false">IF((B12+B13)=0,"",B12/(B12+B13))</f>
@@ -4108,7 +4071,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
@@ -4121,7 +4084,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>278</v>
+        <v>273</v>
       </c>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
@@ -4134,7 +4097,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>279</v>
+        <v>274</v>
       </c>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>

</xml_diff>

<commit_message>
Data handling: drop the no-usable-bucket row
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/deterioration_states/spark/stakeholder/dpd_deterioration_states_reference.xlsx
+++ b/docs/deterioration_states/spark/stakeholder/dpd_deterioration_states_reference.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="275">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="373" uniqueCount="272">
   <si>
     <t xml:space="preserve">DPD deterioration states</t>
   </si>
@@ -796,15 +796,6 @@
   </si>
   <si>
     <t xml:space="preserve">No false payment.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No usable bucket in the window</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Not classified.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Counts against coverage (target 99.9%).</t>
   </si>
   <si>
     <t xml:space="preserve">Latest month older than the scoring date</t>
@@ -3623,7 +3614,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
@@ -3750,17 +3741,6 @@
       </c>
       <c r="C13" s="9" t="s">
         <v>258</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="56" t="s">
-        <v>259</v>
-      </c>
-      <c r="B14" s="9" t="s">
-        <v>260</v>
-      </c>
-      <c r="C14" s="9" t="s">
-        <v>261</v>
       </c>
     </row>
   </sheetData>
@@ -3798,12 +3778,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -3819,28 +3799,28 @@
         <v>11</v>
       </c>
       <c r="B4" s="7" t="s">
+        <v>261</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>262</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>263</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>262</v>
+      </c>
+      <c r="F4" s="7" t="s">
         <v>264</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="G4" s="7" t="s">
+        <v>262</v>
+      </c>
+      <c r="H4" s="7" t="s">
         <v>265</v>
       </c>
-      <c r="D4" s="7" t="s">
-        <v>266</v>
-      </c>
-      <c r="E4" s="7" t="s">
-        <v>265</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>267</v>
-      </c>
-      <c r="G4" s="7" t="s">
-        <v>265</v>
-      </c>
-      <c r="H4" s="7" t="s">
-        <v>268</v>
-      </c>
       <c r="I4" s="7" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4020,7 +4000,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="23" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="B12" s="59" t="n">
         <f aca="false">SUM(B5:B11)</f>
@@ -4041,7 +4021,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="60" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="B13" s="61"/>
       <c r="D13" s="61"/>
@@ -4050,7 +4030,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="23" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="B14" s="62" t="str">
         <f aca="false">IF((B12+B13)=0,"",B12/(B12+B13))</f>
@@ -4071,7 +4051,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
@@ -4084,7 +4064,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
@@ -4097,7 +4077,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>

</xml_diff>

<commit_message>
Data handling: drop the stale-latest-month row
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/deterioration_states/spark/stakeholder/dpd_deterioration_states_reference.xlsx
+++ b/docs/deterioration_states/spark/stakeholder/dpd_deterioration_states_reference.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="373" uniqueCount="272">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="269">
   <si>
     <t xml:space="preserve">DPD deterioration states</t>
   </si>
@@ -796,15 +796,6 @@
   </si>
   <si>
     <t xml:space="preserve">No false payment.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Latest month older than the scoring date</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Flagged.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Classified on the history we have.</t>
   </si>
   <si>
     <t xml:space="preserve">Results</t>
@@ -3614,7 +3605,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
@@ -3730,17 +3721,6 @@
       </c>
       <c r="C12" s="9" t="s">
         <v>255</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="56" t="s">
-        <v>256</v>
-      </c>
-      <c r="B13" s="9" t="s">
-        <v>257</v>
-      </c>
-      <c r="C13" s="9" t="s">
-        <v>258</v>
       </c>
     </row>
   </sheetData>
@@ -3778,12 +3758,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -3799,28 +3779,28 @@
         <v>11</v>
       </c>
       <c r="B4" s="7" t="s">
+        <v>258</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>259</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>260</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>259</v>
+      </c>
+      <c r="F4" s="7" t="s">
         <v>261</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="G4" s="7" t="s">
+        <v>259</v>
+      </c>
+      <c r="H4" s="7" t="s">
         <v>262</v>
       </c>
-      <c r="D4" s="7" t="s">
-        <v>263</v>
-      </c>
-      <c r="E4" s="7" t="s">
-        <v>262</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>264</v>
-      </c>
-      <c r="G4" s="7" t="s">
-        <v>262</v>
-      </c>
-      <c r="H4" s="7" t="s">
-        <v>265</v>
-      </c>
       <c r="I4" s="7" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4000,7 +3980,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="23" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="B12" s="59" t="n">
         <f aca="false">SUM(B5:B11)</f>
@@ -4021,7 +4001,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="60" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="B13" s="61"/>
       <c r="D13" s="61"/>
@@ -4030,7 +4010,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="23" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="B14" s="62" t="str">
         <f aca="false">IF((B12+B13)=0,"",B12/(B12+B13))</f>
@@ -4051,7 +4031,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="2" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
@@ -4064,7 +4044,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="B17" s="2"/>
       <c r="C17" s="2"/>
@@ -4077,7 +4057,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>

</xml_diff>